<commit_message>
Add STORM-006 to STORM-010 to Storm Case Database
Processed five FOS storm decisions:
  STORM-006 DRN-2560515  Royal & Sun Alliance  Not Upheld
  STORM-007 DRN-2737383  Liverpool Victoria    Upheld
  STORM-008 DRN-2788212  Lloyds Bank           Not Upheld
  STORM-009 DRN-2877529  Lloyds Bank           Not Upheld
  STORM-010 DRN-2926734  Fairmead              Upheld

Database now contains 10 storm cases (STORM-001 to STORM-010).
28 PDFs remain (STORM-011 to STORM-038).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Storm_Case_Database.xlsx
+++ b/knowledge/case-databases/Storm_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1128,6 +1128,531 @@
         </is>
       </c>
     </row>
+    <row r="7" ht="120" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>STORM-006</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>DRN-2560515</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Royal &amp; Sun Alliance Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>8 Jun 2021</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Caravan roof seal failure claimed as storm damage; three repairers all attributed cause to general weathering or design fault; no visible storm-consistent damage such as lifted or broken roof panels; Q2 failed</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Caravan roof ridge seal and bolt hole failure — seals attributed to general weathering or design fault by all three repairers; no lifted or broken roof panels consistent with storm</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Static caravan</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Three repairers assessed the caravan — one said seals failed due to general weathering; RSA's specialist initially noted storm or design fault but later concluded design fault as there was no visible storm damage to the roof; no evidence of lifted or broken roof panels</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>RSA relied on three concurrent repairer assessments all attributing cause to weathering or design fault; Mrs L argued that less water ingress would be expected from a design fault, but RSA's file showed the site owner confirmed water damage was getting worse; no independent expert evidence submitted to challenge the repairer findings</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; RSA's decision to decline confirmed as fair and reasonable; RSA not at fault for delays in obtaining quotes as site owner took three months; no evidence RSA pressured its specialist into changing position; no award</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P7" s="5" t="inlineStr">
+        <is>
+          <t>All three storm questions must be answered yes; Q2 failed — no evidence of damage consistent with a storm such as lifted or broken roof panels; three concurrent repairer opinions all attributing cause to weathering or design fault is highly persuasive in the absence of independent counter-evidence; an insurer is entitled to rely on concurrent expert opinions to decline</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>Independent expert report challenging the three repairer assessments; photographs showing storm-consistent structural damage such as lifted or broken roof panels; evidence ruling out general weathering and design fault as the cause</t>
+        </is>
+      </c>
+      <c r="R7" s="5" t="inlineStr">
+        <is>
+          <t>Storm conditions present (Q1 yes); no evidence of damage consistent with storm — no lifted or broken roof panels (Q2 no); all three repairers attributed cause to general weathering or design fault; RSA's specialist changed its initial equivocal position to design fault after confirming no visible storm damage; Mrs L's argument that less ingress would be expected from a design fault was contradicted by the site owner confirming damage was worsening; no evidence RSA pressured its contractor to change position; Q2 answered no means Q3 not reached</t>
+        </is>
+      </c>
+      <c r="S7" s="5" t="inlineStr">
+        <is>
+          <t>Where three independent repairers all attribute damage to weathering or design fault, an insurer can rely on this concurrence to decline without storm causation being established; absence of lifted or broken structural panels is a key negative indicator for Q2; a policyholder's subjective expectation about the degree of ingress from a design fault does not override concurrent expert physical assessments</t>
+        </is>
+      </c>
+      <c r="T7" s="5" t="inlineStr">
+        <is>
+          <t>IF three_or_more_repairers_attribute_damage_to_weathering_or_design_fault AND no_lifted_or_broken_roof_panels THEN storm_q2 = no AND claim = not_established; IF insurer_has_concurrent_expert_opinions AND policyholder_has_no_independent_expert_evidence THEN insurer_evidence = decisive</t>
+        </is>
+      </c>
+      <c r="U7" s="4" t="inlineStr">
+        <is>
+          <t>DRN-2560515.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="120" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>STORM-007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>DRN-2737383</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Liverpool Victoria Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>7 May 2021</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Storm damage to residential roof in February 2020; LV declined external damage (tiles, hips, felt, lead flashing) citing wear and tear but based its exclusion on a different roof area from that being claimed for; repair contractor confirmed good overall roof condition and storm causation; FOS upheld</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Roof tiles, hips and felt damaged with lead flashing lifted — contractor confirmed lifted tiles and ripped felt caused by gale force winds in the claimed area; LV inspected a different roof section and applied exclusion incorrectly to uninspected area</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Partial</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>LV's contractor found age-related deterioration, historic repairs and lead flashing used as a substitute for hip tiles in the inspected areas; LV relied on these findings and Google Street View images to conclude wear and tear and poor workmanship; declined external damage while accepting internal damage and contents</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>LV relied on ground-level contractor report and Google Street View images showing deterioration on inspected areas of the roof; Mr H's contractor confirmed the claimed area showed good overall roof condition (lathes and underfelt very good) with lifted tiles and ripped felt consistent with storm damage from gale force winds; LV's own agent who inspected internal damage confirmed water ingress was fresh and not longstanding; repair invoice included chimney works not connected to storm damage, complicating settlement quantum</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>Upheld — LV must deal with Mr H's storm damage claim for the affected roof areas he claimed for and had repaired; add 8% simple interest to any cash settlement from date of payment to date of settlement; pay Mr H a further £100 compensation in addition to the £100 already paid for delays</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>An insurer must inspect the specific area of roof being claimed for before applying a wear and tear or poor workmanship exclusion; relying on the condition of a different and unrelated roof section to decline a storm claim for an uninspected area is not fair or reasonable; where the insurer's own agent confirms water ingress was fresh and not longstanding, this undermines a maintenance or wear and tear defence; an insurer that fails to inspect the damaged area cannot demonstrate the exclusion applies to that area</t>
+        </is>
+      </c>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>Itemised repair invoice breaking down storm-related costs from non-storm elements (chimney and other non-storm works); physical inspection by LV of the specific roof area where storm damage was claimed</t>
+        </is>
+      </c>
+      <c r="R8" s="3" t="inlineStr">
+        <is>
+          <t>Storm conditions agreed (Q1 yes); damage type — lifted tiles, ripped felt, lifted lead flashing and resultant internal water ingress — consistent with storm damage (Q2 yes); LV inspected only from ground level and did not view the claimed area, instead relying on condition of a different roof section to apply the exclusion — exclusion not shown to apply to the claimed area (Q3 — LV failed to discharge burden); Mr H's contractor confirmed good overall condition with storm-consistent damage in the claimed area; LV's own agent confirmed ingress was fresh not longstanding, inconsistent with longstanding maintenance failure</t>
+        </is>
+      </c>
+      <c r="S8" s="3" t="inlineStr">
+        <is>
+          <t>Inspections must cover the specific area of damage being claimed for; applying a wear and tear exclusion to an uninspected roof section based on the condition of a different area is not fair and will not be upheld by FOS; where a contractor confirms good overall roof condition and storm-consistent damage in the claimed area, and the insurer's own agent reports fresh ingress, storm causation is established for that area; repair invoices covering mixed storm and non-storm works must be itemised before settlement</t>
+        </is>
+      </c>
+      <c r="T8" s="3" t="inlineStr">
+        <is>
+          <t>IF insurer_inspected_different_roof_area AND applied_exclusion_to_uninspected_claimed_area THEN exclusion_not_shown_to_apply AND outright_decline_not_fair; IF contractor_confirms_good_roof_condition_in_claimed_area AND insurers_own_agent_confirms_fresh_ingress THEN storm_causation_established_for_claimed_area; IF repair_invoice_contains_non_storm_works THEN require_itemised_breakdown_before_settlement</t>
+        </is>
+      </c>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
+          <t>DRN-2737383.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="120" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>STORM-008</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>DRN-2788212</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Lloyds Bank General Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>11 Jun 2021</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Water ingress through roof during storm; policyholder carried out urgent repairs and builder disposed of damaged materials before insurer could inspect; no photographic evidence of pre-repair damage; builder statement alone insufficient to establish Q2 or Q3; claim declined for failure to substantiate loss</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Roof water ingress — nature of storm damage unknown as repairs were completed and damaged materials disposed of before inspection; storm conditions confirmed but damage pattern could not be assessed</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Repairs completed and damaged materials disposed of before Lloyds could inspect; photos provided only showed completed repairs not pre-repair damage; builder gave conflicting reasons when Lloyds spoke to him; Lloyds could not validate Q2 or Q3 without physical evidence</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>Mr and Mrs H provided photos of completed roof repairs and a builder email stating the roof was in good condition and damage was wind-caused; Lloyds argued photos showed only completed work, builder gave conflicting reasons when contacted, and damaged sections had been disposed of; FOS agreed builder's statement alone was insufficient and that Q2 and Q3 could not be answered without physical evidence of the pre-repair damage</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; Lloyds acted fairly and within policy terms in declining; policyholder failed to provide sufficient evidence to establish storm causation; no award</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P9" s="5" t="inlineStr">
+        <is>
+          <t>Policyholder must not carry out non-emergency repairs or dispose of damaged items before the insurer has had a chance to inspect; storm conditions alone (Q1) are insufficient without evidence to establish Q2 and Q3; a builder's statement without photographic or physical evidence of pre-repair damage does not prove storm causation; a well-maintained roof should withstand all but the most severe weather and Q2 requires evidence to assess this</t>
+        </is>
+      </c>
+      <c r="Q9" s="5" t="inlineStr">
+        <is>
+          <t>Photographs of the damaged roof taken before repair commenced; damaged roofing materials (tiles, felt, etc.) retained for inspection; independent inspection of the roof before repair; explanation of the conflicting reasons given by the builder to Lloyds</t>
+        </is>
+      </c>
+      <c r="R9" s="5" t="inlineStr">
+        <is>
+          <t>Storm conditions present (Q1 yes); Q2 and Q3 could not be answered as repairs were completed and materials disposed of before Lloyds could inspect — no pre-repair photographs and no physical evidence remained; builder gave conflicting reasons to Lloyds; policy required policyholder to preserve evidence and notify insurer before non-emergency repairs; builder could have photographed the damage before starting work; Lloyds acted fairly in declining on the evidence available</t>
+        </is>
+      </c>
+      <c r="S9" s="5" t="inlineStr">
+        <is>
+          <t>Policyholders who carry out urgent storm repairs must photograph all damage and retain damaged materials before work commences; a builder carrying out repairs without documenting the pre-repair state removes the insurer's ability to validate Q2 and Q3; insurers should communicate evidence-preservation obligations clearly at first notification; a builder's verbal or written statement without corroborating physical evidence is insufficient to establish storm causation</t>
+        </is>
+      </c>
+      <c r="T9" s="5" t="inlineStr">
+        <is>
+          <t>IF repairs_completed_before_inspection AND damaged_materials_disposed_of AND no_pre_repair_photographs THEN claim_evidence_insufficient AND Q2_Q3_cannot_be_answered AND decline_reasonable; IF only_evidence_is_builder_statement AND no_physical_evidence_of_storm_damage THEN storm_causation_not_established</t>
+        </is>
+      </c>
+      <c r="U9" s="4" t="inlineStr">
+        <is>
+          <t>DRN-2788212.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="120" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>STORM-009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>DRN-2877529</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Lloyds Bank General Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>21 Jul 2021</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Chimney stack water ingress following storms Clara and Denis in February 2020; surveyor found no displaced tiles or render and attributed damage to natural breakdown of flaunching; contractor estimate made no reference to storm damage; external chimney claim declined, internal bedroom damage accepted; FOS not upheld</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Chimney stack — deterioration of flaunching with no displaced tiles or render; chimney caps undisturbed; water entered through everyday weathering not a one-off storm event</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Partial</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Surveyor found no visible storm damage to the chimney — no displaced tiles or render, caps still in place, nothing disturbed by wind; flaunching deterioration attributed to natural breakdown of materials; contractor estimate for chimney repairs made no reference to storm damage</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Lloyds relied on surveyor report and photos showing no storm-consistent physical indicators on the chimney and a contractor estimate not referencing storm damage; Mrs C said the damp in the bedroom wall worsened considerably after storms Clara and Denis and that she had always maintained the chimney; FOS agreed with Lloyds that absence of physical storm indicators was decisive regardless of the timing of observed damp worsening</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; Lloyds correctly declined external chimney damage as not consistent with storm; Lloyds had already accepted internal bedroom damage; no award on the chimney claim</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>Q2 requires damage to be consistent with storm-typical damage; where a surveyor finds no displaced tiles or render and chimney caps remain in place and undisturbed, Q2 is answered no; deterioration of flaunching is a maintenance issue not a storm peril; a policyholder observing damp worsen after storms does not establish storm causation where physical evidence shows no storm-consistent structural disturbance; contractor estimates that do not reference storm damage are a significant negative indicator</t>
+        </is>
+      </c>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>Independent expert report attributing chimney damage to storm; photographs showing displaced tiles, render failure or chimney cap disturbance; evidence of chimney condition immediately before the storms</t>
+        </is>
+      </c>
+      <c r="R10" s="3" t="inlineStr">
+        <is>
+          <t>Storm conditions present (Q1 yes); surveyor found no displaced tiles or render, chimney caps still in place and nothing disturbed by wind (Q2 no); contractor estimate gave no reference to storm damage; FOS agreed external damage was not consistent with storm; Mrs C's observation that damp worsened after the storms did not override physical evidence showing no storm indicators; Lloyds correctly applied the three-question framework and declined the external chimney claim; internal bedroom damage already accepted</t>
+        </is>
+      </c>
+      <c r="S10" s="3" t="inlineStr">
+        <is>
+          <t>Worsening damp after storms is not conclusive of storm causation — always check for physical storm indicators such as displaced tiles, disturbed render or lifted chimney caps; where a surveyor finds flaunching deterioration with no structural disturbance, Q2 is answered no; a contractor estimate that does not reference storm damage is a significant negative indicator; chimneys are a common source of gradual water ingress and require clear physical storm evidence to distinguish from ongoing deterioration</t>
+        </is>
+      </c>
+      <c r="T10" s="3" t="inlineStr">
+        <is>
+          <t>IF surveyor_finds_no_displaced_tiles_or_render AND chimney_caps_undisturbed THEN storm_q2 = no AND damage = weathering_not_storm; IF contractor_estimate_contains_no_storm_damage_reference AND surveyor_attributes_damage_to_natural_breakdown THEN insurer_decline_of_chimney = reasonable; IF policyholder_reports_damp_worsening_after_storm AND no_physical_storm_indicators THEN temporal_correlation_insufficient_to_establish_causation</t>
+        </is>
+      </c>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>DRN-2877529.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="120" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>STORM-010</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>DRN-2926734</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Fairmead Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>12 Aug 2021</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Water ingress through roof in October 2020; Fairmead outright declined citing no storm conditions on the precise date of loss; FOS found 49mph gusts on 25 September 2020 (within policy's 47mph definition) shortly before the damage; property in exposed coastal location; insurer directed to reconsider with full inspection</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Roof water ingress — lifted tiles visible in policyholder photographs; dominant cause not determined as Fairmead declined without inspection</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Fairmead said weather conditions on 3 October 2020 (reported date of loss) did not reach storm force as defined in the policy (gusts of at least 47mph); declined outright on this basis without inspecting the property or assessing Q2 or Q3</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>Fairmead relied on weather records for the specific date of loss showing sub-47mph winds; Ms B provided photos showing lifted tiles and internal water damage; FOS reviewed broader weather records and found 49mph gusts on 25 September 2020 shortly before the loss meeting the policy storm definition; Fairmead's own claim notes acknowledged the property was in an exposed coastal location which could mean actual conditions exceeded nearest weather station readings</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>Upheld — Fairmead directed to reconsider Ms B's storm damage claim in line with remaining policy terms including arranging a physical inspection; pay Ms B £100 compensation for distress caused by incorrect outright decline; if Ms B remains dissatisfied after reconsideration she may bring a new complaint</t>
+        </is>
+      </c>
+      <c r="N11" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P11" s="5" t="inlineStr">
+        <is>
+          <t>Weather records must be checked over the period leading up to the date of loss, not only on the precise reported date; a policy storm definition of 47mph gusts is met by 49mph gusts recorded shortly before the loss; an exposed coastal location means actual conditions at the property may exceed nearest weather station readings; outright declining without physical inspection when storm conditions did occur in the relevant period is not fair or reasonable; an insurer must assess all three questions before declining</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="inlineStr">
+        <is>
+          <t>Physical inspection of roof and internal damage by Fairmead; independent expert report on whether storm or gradual deterioration was the dominant cause; weather data specific to the exposed coastal location rather than the nearest weather station</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>Policy defined storm as 47mph gusts; weather records showed 49mph on 25 September 2020 shortly before the loss — Q1 met on the broader weather record; Ms B's photos showed lifted tiles and internal water damage consistent with storm damage (Q2 provisionally yes); Fairmead declined outright without inspecting so Q3 could not be assessed — dominant cause undetermined; Fairmead incorrectly assessed storm conditions only on the precise date of loss rather than the period leading up to it; exposed coastal location acknowledged by Fairmead itself as a relevant factor; directed to reconsider with full inspection and pay £100 compensation</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>Weather records must be reviewed over the relevant period before the date of loss, not just the precise date reported — storm conditions occurring days before visible damage can still satisfy Q1; an insurer that declines solely on weather records without inspecting the property cannot assess Q2 or Q3 and risks an incorrect outright decline; an exposed coastal location is a material factor requiring consideration when comparing weather station data to actual property conditions; always inspect before declining when storm conditions occurred in the relevant period</t>
+        </is>
+      </c>
+      <c r="T11" s="5" t="inlineStr">
+        <is>
+          <t>IF weather_records_show_storm_conditions_in_period_before_date_of_loss AND insurer_checked_only_exact_date_reported THEN storm_q1_assessment_incomplete AND outright_decline_not_justified; IF insurer_declined_without_inspection AND storm_conditions_occurred_in_relevant_period THEN insurer_must_reconsider_and_inspect; IF property_in_exposed_location AND weather_station_readings_near_threshold THEN actual_conditions_may_exceed_station_readings</t>
+        </is>
+      </c>
+      <c r="U11" s="4" t="inlineStr">
+        <is>
+          <t>DRN-2926734.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add STORM-011 to STORM-015 to Storm Case Database
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Storm_Case_Database.xlsx
+++ b/knowledge/case-databases/Storm_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1653,6 +1653,531 @@
         </is>
       </c>
     </row>
+    <row r="12" ht="120" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>STORM-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>DRN-2926772</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>National Farmers' Union Mutual Insurance Society Limited</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>26 Oct 2021</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Second storm damage claim for porch roof water ingress in August 2020; NFU's loss adjuster found no storm indicators — only chipped tiles, loose mortar in lead valleys and gapping lead flashing attributed to wear and tear and poor workmanship; policyholder's expert report asserted storm damage but contained no photographs and could not displace NFU's photographic evidence; Q2 failed</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Porch roof — chipped tiles, loose mortar sitting in lead valleys and gapping lead flashing where flashing had come away from mortar; loss adjuster found no missing tiles, damaged roofing felt or punctured lead valleys consistent with storm</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>NFU's loss adjuster found no signs of storm damage — photos showed chipped tiles, loose mortar in lead valleys and gapping lead flashing; findings attributed to wear and tear and poor workmanship; damage pattern not consistent with storm-typical indicators such as missing tiles, damaged felt or punctured lead valleys</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>NFU relied on its loss adjuster's report and photographic evidence showing wear and tear and poor workmanship; Ms R provided a builder's report asserting storm and rain caused damage including missing tiles and damaged felt, but the report contained no photographs; FOS found the available photos did not show the storm damage Ms R's expert described; minor errors Ms R identified in NFU's report were found not material enough to undermine its overall findings</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; NFU's decision to decline confirmed as fair and reasonable; Ms R's expert report without photographs could not displace NFU's photographic evidence; NFU's handling of the first claim and request for repair estimates also found reasonable; no award</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>Q2 failed — photos showed no missing tiles, damaged felt or punctured lead valleys consistent with storm; a policyholder's expert report without photographs cannot displace an insurer's expert evidence supported by photos; minor errors in a loss adjuster's report do not undermine its conclusions where photographs support the findings; policy excludes damage happening gradually and damage caused by faulty workmanship</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>Photographs from Ms R's expert showing missing tiles, damaged roofing felt and punctured lead valleys; independent expert inspection with physical evidence to contradict NFU's photographic findings; evidence ruling out wear and tear and poor workmanship as the cause</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>Q1 disputed but FOS addressed Q2 first; Q2 — photos showed chipped tiles, loose mortar in lead valleys and gapping lead flashing consistent with wear and tear and poor workmanship; no missing tiles, damaged felt or punctured lead valleys visible; Ms R's builder's report claimed tiles had come off in high winds and felt was damaged but provided no photographs and could not displace NFU's photographic evidence; minor report errors not material; Q2 answered no so Q3 not reached; NFU's handling of repair estimates and the first claim found reasonable on the call recording evidence</t>
+        </is>
+      </c>
+      <c r="S12" s="3" t="inlineStr">
+        <is>
+          <t>Where an insurer has photographic evidence consistent with its expert's findings of wear and tear, a policyholder's expert report without photographs will not displace that evidence; chipped tiles and loose mortar in lead valleys without missing or dislodged structural elements indicate wear and tear not storm; a loss adjuster report's immaterial errors do not invalidate its conclusions where photos support them; policy exclusions for gradual damage and faulty workmanship apply concurrently with a storm Q2 failure</t>
+        </is>
+      </c>
+      <c r="T12" s="3" t="inlineStr">
+        <is>
+          <t>IF insurer_expert_report_supported_by_photographs AND policyholder_expert_report_has_no_photographs THEN insurer_evidence_prevails; IF photos_show_chipped_tiles_and_loose_mortar AND no_missing_tiles_or_damaged_felt_or_punctured_lead_valleys THEN storm_q2 = no AND damage = wear_and_tear; IF loss_adjuster_report_has_minor_errors AND photos_support_overall_conclusions THEN report_errors_not_material_and_conclusions_stand</t>
+        </is>
+      </c>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>DRN-2926772.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="120" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>STORM-012</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3173328</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>4 Jan 2022</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Buildings insurance storm damage claim for water damage to airing cupboard and suspected dropped roof profile; Aviva's surveyor found no storm damage — facias and roof tiles undamaged and in place, chimney flaunching in poor condition; airing cupboard staining attributed to gradual aging not a one-off storm event; £100 delay compensation pre-paid by Aviva confirmed adequate by FOS</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Roof — staining in airing cupboard and suspected dropped roof profile; surveyor found no damage to soffits, facias or roof tiles; all tiles in place; chimney flaunching and pointing in poor condition; staining attributed to aging and gradual deterioration not a storm event</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Aviva's surveyor found no damage to soffits or facias and all roof tiles were in place; staining in the airing cupboard attributed to aging and gradual deterioration rather than a one-off storm event; any problems identified pre-existed the bad weather; independent roofer's photos reviewed by Aviva still showed wear and tear not storm damage</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>Aviva relied on its surveyor's report showing no storm indicators and on its review of Miss D's roofer's photos which it still found showed wear and tear not storm damage; Miss D's roofer said a section of tiles was lifting during high winds; FOS agreed Aviva was entitled to rely on its surveyor's finding that problems pre-existed the storm; surveyor found moss growth and chimney flaunching and pointing in poor condition as further indicators of gradual deterioration</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; Aviva's decision to decline confirmed as fair and reasonable; £100 compensation pre-paid by Aviva for delay in communicating findings confirmed as the right amount — the sort of amount FOS would have ordered if not already paid; no further award</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P13" s="5" t="inlineStr">
+        <is>
+          <t>Q2 and Q3 not satisfied; where a surveyor finds no damage to soffits, facias or roof tiles and attributes airing cupboard staining to gradual aging rather than a one-off event, an insurer is entitled to rely on that opinion to decline; a roofer's report that tiles were lifting during high winds does not override a surveyor's finding of no storm damage where the insurer finds problems pre-existed the storm; delay in communicating claim decisions warrants compensation independently of the coverage decision</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="inlineStr">
+        <is>
+          <t>Structural evidence of sudden storm-caused damage rather than gradual deterioration; photographs showing tiles actually missing or structurally displaced rather than merely lifting; evidence distinguishing the property's pre-storm condition from its post-storm condition</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>Q1 — storm conditions accepted by Aviva; Q2 and Q3 — surveyor found no damage to soffits or facias, all roof tiles in place, chimney flaunching in poor condition; staining in airing cupboard consistent with gradual aging not a one-off storm event; Miss D's roofer said tiles lifting in high winds but Aviva found problems pre-existed the storm and FOS agreed the insurer was entitled to rely on its surveyor; £100 delay compensation pre-paid by Aviva confirmed as appropriate — FOS would have required the same amount</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>A surveyor finding all roof tiles in place and no soffit or fascia damage is strong evidence against a storm claim; gradual staining in an interior space is likely deterioration unless a one-off event can be evidenced; delay in communicating claim decisions should be compensated even when the coverage decline is upheld; pre-existing problems identified at inspection defeat storm causation even where storm conditions occurred</t>
+        </is>
+      </c>
+      <c r="T13" s="5" t="inlineStr">
+        <is>
+          <t>IF surveyor_finds_no_damage_to_soffits_facias_or_tiles AND interior_staining_attributed_to_gradual_aging THEN storm_q2_q3 = not_satisfied AND decline_reasonable; IF insurer_delayed_communicating_decision AND caused_policyholder_stress THEN compensate_for_delay_regardless_of_coverage_outcome; IF policyholder_roofer_says_tiles_lifting AND insurer_surveyor_finds_problems_preexisted THEN insurer_entitled_to_rely_on_surveyor_and_decline</t>
+        </is>
+      </c>
+      <c r="U13" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3173328.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="120" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>STORM-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3211590</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>26 Jan 2022</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Storm damage to residential roof in December 2020; loss adjuster and independent assessor both found the original construction of the verge tiles was inadequate and this was the dominant cause; storm damage claim declined under faulty workmanship/defective design exclusion; Aviva separately accepted falling debris damage to single storey roof under accidental damage</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Upper roof verge tiles — poor original construction and inadequate fitting identified as dominant cause; previous repointing repairs done by cementing over existing mortar rather than removing it first; debris dislodged from double storey roof damaged the single storey roof below</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Partial</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Loss adjuster and independent assessor both concluded the original construction of the verge tiles was inadequate on both the double and single storey roofs; repointing repairs four years prior done incorrectly; damage would not have occurred but for the poor original construction and fitting of verge tiles; policy excludes faulty workmanship, defective design and defective materials</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>Aviva relied on its loss adjuster and an independent assessor who both concluded poor original construction of verge tiles was the dominant cause; Miss G argued the assessors focused on previously repaired areas she was not claiming for and that the verges she was claiming were differently constructed; Miss G provided contractor advice that verge tiles are designed to be held by the weight of tiles above with fixings on every 2nd or 3rd row; FOS found the independent assessor's conclusions covered the overall construction of both roofs and were not displaced by contractor statements</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold storm damage claim; Aviva's decision confirmed as reasonable; Aviva had properly accepted falling tiles onto the single storey roof under accidental damage; no additional award on the storm damage claim</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>Q3 failed — where two expert assessments (loss adjuster and independent assessor) both conclude poor original construction was the dominant cause, storm is not the main cause even if storm conditions occurred; policy exclusion for faulty workmanship and defective design applies; accepting consequential falling debris under accidental damage while declining the storm claim is a valid partial position; the policyholder must produce evidence of equal weight to contradict expert assessors</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>Independent evidence of equal weight contradicting both assessors' findings on verge tile construction; physical evidence demonstrating the verge tiles at the specific claimed location were adequately constructed before the storm; evidence ruling out poor original construction as the dominant cause</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="inlineStr">
+        <is>
+          <t>Q1 — storm conditions accepted by Aviva; Q2 — possibly consistent with storm (FOS noted this without deciding definitively); Q3 — loss adjuster and independent assessor both found the damage would not have occurred but for poor original construction and fitting of verge tiles on both roofs; Miss G's argument that assessors focused on different roof areas not accepted as the assessor's conclusions covered overall construction; no evidence of equal weight to contradict; Aviva's acceptance of falling debris under accidental damage was a proper and fair partial position</t>
+        </is>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>Where two expert assessments both attribute damage to poor original construction, a Q3 failure is well-founded even where the policyholder produces contractor statements to the contrary; accepting consequential damage under accidental damage while declining the main storm claim is a valid and fair approach; policyholders contesting the geographic focus of assessors' reports must produce evidence that the area they are specifically claiming for was differently and adequately constructed</t>
+        </is>
+      </c>
+      <c r="T14" s="3" t="inlineStr">
+        <is>
+          <t>IF two_expert_assessments_both_attribute_damage_to_poor_original_construction AND no_contradicting_evidence_of_equal_weight THEN storm_q3 = no AND decline_reasonable; IF policy_excludes_faulty_workmanship_and_defective_design AND experts_conclude_poor_construction_dominant THEN exclusion_applies; IF insurer_accepts_consequential_damage_under_accidental_damage_while_declining_storm THEN partial_acceptance_valid_and_fair</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3211590.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="120" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>STORM-014</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3295758</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>16 Jun 2022</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Retaining and boundary wall collapse at rear of property attributed to Storm Dennis in February 2020; structural engineer found the retaining wall too thin and inadequate for the three-metre retained height and that the boundary wall had been deteriorating hidden from view; gradual deterioration not storm was the dominant cause; decline confirmed</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Retaining wall (mix of stone, brick and concrete block) collapsed into footpath — structural engineer found wall very thin and inadequate for the three-metre retained height; boundary wall hidden behind it in disrepair and undermined by the newer retaining wall over time; gradual deterioration not a storm event</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Structural engineer's report found the retaining wall very thin and inadequate for the retained height — described as surprising it had lasted as long as it had; remaining wall section bowed and cracked; the boundary wall behind had been undermined by the retaining wall and was in disrepair hidden from view; damage was caused by gradual deterioration not a storm event</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>Aviva relied on the structural engineer's report showing the retaining wall was too thin and inadequate, the remaining section bowed and cracked, and the boundary wall in disrepair hidden behind hedging; Mrs V argued the collapse was caused by Storm Dennis and that her garden sloped; FOS agreed the structural evidence showed gradual deterioration and structural inadequacy rather than storm as the dominant cause</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; Aviva's decision to decline confirmed as fair and reasonable; policy exclusion for damage happening gradually applied correctly; other policy sections (flooding, subsidence/landslip) also considered and found inapplicable; no award; question of retaining wall ownership noted as a matter Mrs V could pursue separately</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>Q2 and Q3 failed — wall collapse from a structurally inadequate and gradually deteriorating structure is not typical storm damage and storm was not the main cause; policy general exclusion for damage happening gradually over time explicitly lists boundary walls as prone to wear and tear; an inadequate structure described as surprising it lasted so long fails Q3 even where strong storm conditions (Storm Dennis, 70mph peak gust) occurred; subsidence/landslip cover requires the home to be affected — boundary walls alone do not qualify</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>Evidence that the wall collapse was a sudden one-off event rather than gradual deterioration; independent structural report attributing the collapse primarily to the storm rather than structural inadequacy; evidence that the wall was adequately constructed and maintained before the storm</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="inlineStr">
+        <is>
+          <t>Q1 — Storm Dennis 13–19 February 2020, peak gust 70mph, storm conditions confirmed; Q2 — wall collapse could be storm-consistent but structural evidence showed gradual deterioration; Q3 — structural engineer found retaining wall too thin and inadequate for three-metre height and surprising it had lasted so long; remaining section bowed and cracked; boundary wall undermined by retaining wall over time; storm not the main cause; policy exclusion for gradual damage applied; boundary walls listed as wear-and-tear examples; flooding and subsidence/landslip sections considered and found inapplicable</t>
+        </is>
+      </c>
+      <c r="S15" s="5" t="inlineStr">
+        <is>
+          <t>Even where strong storm conditions are confirmed (Storm Dennis 70mph), a wall with structural inadequacy and pre-existing gradual deterioration fails Q3; boundary walls are explicitly identified in many policies as prone to wear and tear — always check the general exclusion language; where two walls are involved (boundary and retaining), both must be assessed individually against the storm questions; always check all relevant policy sections when declining to ensure no alternative peril applies</t>
+        </is>
+      </c>
+      <c r="T15" s="5" t="inlineStr">
+        <is>
+          <t>IF structural_engineer_finds_wall_too_thin_and_inadequate AND remaining_section_bowed_and_cracked THEN storm_q3 = no AND damage = gradual_deterioration; IF policy_lists_boundary_walls_as_wear_and_tear_example AND gradual_deterioration_confirmed THEN exclusion_applies; IF storm_conditions_confirmed AND structure_was_pre_existing_inadequate AND surprising_it_lasted_so_long THEN storm_not_main_cause AND decline_reasonable</t>
+        </is>
+      </c>
+      <c r="U15" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3295758.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="120" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>STORM-015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3574617</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Lloyds Bank General Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>13 Sep 2022</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Storm damage claim for roof and bay window; Lloyds initially assessed remotely and incorrectly applied subsidence; Mr P complained; roof storm damage subsequently accepted and paid with compensation; bay window declined as pre-existing structural distortion not realigned after historic underpinning — storm revealed but did not cause the bay damage; FOS not upheld on bay window</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Bay window structure — historic distortion not realigned after underpinning works many years earlier; Lloyds' expert identified movement away from house as an ongoing connection issue with evidence of historic distortion; storm revealed the structural weakness but did not cause the underlying damage</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Partial</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Lloyds' expert confirmed the bay window damage was an ongoing structural issue with evidence of historic distortion not related to any insured peril; distortion not realigned after underpinning works many years prior; storm identified the weak point but a well-maintained property should withstand all but the most severe conditions; bay window not caused by an insured peril</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>Lloyds relied on an expert report (originally commissioned for subsidence) confirming historic distortion with no insured peril as the cause; Mr P's expert acknowledged pre-existing distortion was not realigned after old underpinning but argued the storm placed shock on the building leaving the bay no longer fit for purpose; FOS preferred Lloyds' expert finding that the storm revealed rather than caused the structural weakness; FOS noted a properly commissioned storm survey would not have changed the conclusion since the cause was already identified</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold bay window complaint; roof damage settlement confirmed as fair; £750 compensation already paid by Lloyds for roof and bay handling failures confirmed as adequate; no additional award</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>Q3 failed for bay window — where an expert identifies pre-existing historic distortion as the ongoing cause and confirms no insured peril caused the damage, storm is not the main cause; storms sometimes reveal existing damage rather than create it; a well-maintained property should withstand all but the most severe conditions; an insurer can rely on a report commissioned under a different peril to identify the actual cause provided the cause is identified; a handling failure in peril assessment does not negate the substantive finding on causation</t>
+        </is>
+      </c>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>Evidence that the bay window was in good structural condition before the storm; evidence that the historic underpinning works had successfully realigned the distortion to the required standard; evidence that no structural issues existed before the named storms occurred</t>
+        </is>
+      </c>
+      <c r="R16" s="3" t="inlineStr">
+        <is>
+          <t>Q1 — three named storms confirmed; Q2 — bay window structure unstable; storm typically dislodges roof not underlying bay structure, but FOS moved to Q3 accepting some storm contribution was possible; Q3 — Lloyds' expert confirmed historic distortion was ongoing and not caused by any insured peril; Mr P's expert acknowledged pre-existing distortion but argued storm caused new structural failure; FOS preferred Lloyds' finding that storm revealed existing weakness; well-maintained property test applied; £750 already paid for handling failures confirmed as adequate; no further award</t>
+        </is>
+      </c>
+      <c r="S16" s="3" t="inlineStr">
+        <is>
+          <t>Where an expert confirms pre-existing historic distortion as the cause and finds no insured peril caused the damage, a storm damage claim fails at Q3 even where some storm contribution occurred; when a storm reveals an existing structural weakness rather than creating damage, the storm is not the main cause; a survey commissioned under the wrong peril can still be used to identify the actual cause of damage; compensation for handling failures does not affect the substantive coverage decision</t>
+        </is>
+      </c>
+      <c r="T16" s="3" t="inlineStr">
+        <is>
+          <t>IF expert_confirms_pre_existing_historic_distortion_as_cause AND no_insured_peril_caused_damage THEN storm_q3 = no AND claim_not_established; IF storm_reveals_pre_existing_structural_weakness THEN storm_not_main_cause AND well_maintained_property_test_applies; IF insurer_surveyed_under_wrong_peril AND expert_still_identified_actual_cause THEN coverage_decision_on_correct_cause_stands</t>
+        </is>
+      </c>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3574617.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add STORM-016 to STORM-020 to Storm Case Database
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Storm_Case_Database.xlsx
+++ b/knowledge/case-databases/Storm_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U16"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2178,6 +2178,531 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="120" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>STORM-016</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3638410</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>AA Underwriting Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>6 Sep 2022</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Garden wall collapsed during storm in November 2021; AA declined citing poor design and faulty workmanship then shifted to vegetation-caused gradual deterioration; no faulty design or workmanship exclusion existed in the policy; vegetation/deterioration argument not evidenced by the surveyor report; FOS confirmed storm conditions and upheld</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Garden wall (residential property boundary structure) — collapsed and found in pieces across the garden during storm; gusts up to 74mph confirmed by FOS weather check; no physical evidence that vegetation had caused gradual mortar breakdown specific to this wall</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>AA's surveyor concluded poor design and faulty workmanship caused the collapse; AA later asserted vegetation had weakened the wall over time through gradual deterioration; neither reason was supported by a policy exclusion (no faulty design/workmanship exclusion) or by specific evidence of vegetative deterioration in the survey report</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>AA relied on surveyor report citing poor design and workmanship and on photos showing vegetation present, arguing vegetation can cause mortar breakdown; Mr and Mrs R argued the wall had stood for years without issue and only came down during this specific storm; FOS checked weather records and found gusts up to 74mph on one tool and up to 60mph on another, both meeting the policy's 55mph storm definition; FOS found AA's vegetation/deterioration argument was a generalisation without specific evidence it applied to this wall</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>Upheld — AA Insurance directed to reimburse the cost Mr and Mrs R incurred having their wall rebuilt, subject to the applicable policy excess, plus 8% simple interest from date of invoice payment to date of settlement</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P17" s="5" t="inlineStr">
+        <is>
+          <t>Where a policy contains no exclusion for faulty design or workmanship, an insurer cannot rely on that reason to decline a storm claim; to invoke a gradual deterioration exclusion the insurer must produce specific evidence that applies to the claimed item — a generalisation that vegetation can cause mortar breakdown is insufficient; if a wall has stood without issue for years, this undermines a poor design or deterioration explanation; wind direction at weather station level is not determinative as ground-level conditions can differ due to terrain and surrounding properties</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>No evidence gaps identified by FOS — all three questions answered yes; the wall's long service history contradicted the poor design theory; AA failed to produce specific evidence that vegetation had caused gradual deterioration of this particular wall</t>
+        </is>
+      </c>
+      <c r="R17" s="5" t="inlineStr">
+        <is>
+          <t>Q1 — FOS weather check found gusts up to 74mph on one tool and up to 60mph on another, both meeting the policy's 55mph (48 knot/Storm Force 10) storm definition; Q2 — wall found collapsed in pieces across the garden, consistent with storm damage; Q3 — no faulty design or workmanship exclusion in the policy so that basis cannot stand; vegetation/deterioration exclusion not demonstrated as the surveyor report addressed only design and workmanship, not gradual wear; AA's wind direction argument rejected as ground-level conditions can differ from weather station readings; all three questions yes, claim valid</t>
+        </is>
+      </c>
+      <c r="S17" s="5" t="inlineStr">
+        <is>
+          <t>Before declining on faulty design or workmanship, verify the policy actually contains that exclusion; to invoke a gradual deterioration exclusion after the initial surveyor report, the insurer must produce specific evidence applicable to the item — not a general statement about what vegetation can do; if a structure has stood for many years without issue, this is relevant evidence against both poor design and gradual deterioration explanations; where one weather data source shows sub-threshold winds, always check additional sources before concluding storm conditions were absent</t>
+        </is>
+      </c>
+      <c r="T17" s="5" t="inlineStr">
+        <is>
+          <t>IF policy_has_no_faulty_design_or_workmanship_exclusion THEN insurer_cannot_decline_on_that_basis; IF insurer_relies_on_gradual_deterioration_exclusion AND evidence_is_only_generalisation_not_specific_to_item THEN exclusion_not_demonstrated AND decline_not_fair; IF multiple_weather_sources_confirm_storm_conditions AND one_source_shows_sub_threshold THEN storm_q1 = yes; IF structure_stood_without_issue_for_years AND insurer_claims_poor_design THEN poor_design_explanation_undermined</t>
+        </is>
+      </c>
+      <c r="U17" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3638410.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="120" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>STORM-017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3643634</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>UK Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>27 Sep 2022</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Storm damage to residential roof November 2021; claim accepted by UKI; dispute concerns cash settlement quantum (storm portion only, excluding pre-existing wear and tear identified by second contractor) and delays including an incorrect decline letter and file closure; FOS confirmed cash settlement fair and £150 total compensation for delays adequate</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Residential roof — storm damage accepted; second contractor inspection found pre-existing wear and tear in addition to storm damage; UKI limited cash settlement to storm-damaged area only (£1,663.39) as wear and tear area excluded under policy</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>N/A — storm damage accepted; UKI limited cash settlement to storm-damaged area only, excluding pre-existing wear and tear area identified by second contractor inspection; cash settlement offered at £1,663.39</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>UKI relied on second contractor's inspection finding mixed storm damage and pre-existing wear and tear, and on the policy's wear and tear exclusion; Mr W provided three independent quotes all indicating pre-existing issues with one saying a full new roof was needed; Mr W argued delays had worsened the roof condition and that UKI should undertake managed repairs not cash settle; FOS found cash settlement was within policy terms and delays were partly attributable to Mr W's rejection of the first contractor</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; UKI's cash settlement for storm damage only (excluding wear and tear area) confirmed as fair within policy terms; policy permits cash settlement and UKI had offered managed repair which Mr W rejected; £150 total compensation already paid by UKI for delays and incorrect decline letter confirmed as adequate; no additional award</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>No — Handling Dispute</t>
+        </is>
+      </c>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>Where an insurer has offered managed repair and the policyholder rejects it, the insurer may switch to a cash settlement at its own-supplier cost rate, which may be less than market rate; when a second inspection reveals pre-existing wear and tear in addition to storm damage, the insurer may limit its cash settlement to the storm portion only in line with the wear and tear exclusion; an insurer is not forced to pay market-rate costs when it has already fulfilled its obligation by offering a repair; delays that are partly attributable to the policyholder's own decisions cannot all be attributed to the insurer</t>
+        </is>
+      </c>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>Breakdown of repair costs separating storm damage from wear and tear; evidence of accelerated roof deterioration caused specifically by UKI's delays rather than the pre-existing wear and tear</t>
+        </is>
+      </c>
+      <c r="R18" s="3" t="inlineStr">
+        <is>
+          <t>Storm damage accepted and a builder appointed within three weeks of notification — no initial delay; Mr W rejected the first contractor (general builders not roofing specialist); second contractor found storm damage and pre-existing wear and tear; UKI incorrectly closed the file causing short Dec–Jan delay; incorrect decline letter sent and later corrected; policy permits cash settlement at own-supplier rate; cash offer of £1,663.39 covers storm damage area only, excluding wear and tear which is policy-excluded; Mr W's three independent quotes all indicated pre-existing issues; £50 for lack of contact and £100 for errors and delay already paid (total £150) confirmed as fair compensation</t>
+        </is>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>When a second inspection reveals mixed storm and wear and tear damage, a cash settlement limited to the storm portion only is valid under a wear and tear exclusion; if the policyholder rejects the insurer's initial repair offer, the insurer may offer cash settlement at its own-supplier rate; not all delays in a claim can be attributed to the insurer — some result from the policyholder's own decisions; an incorrect decline letter that is promptly corrected does not require uplift in compensation beyond the insurer's existing offer if that offer is adequate</t>
+        </is>
+      </c>
+      <c r="T18" s="3" t="inlineStr">
+        <is>
+          <t>IF insurer_offered_managed_repair AND policyholder_rejected_it AND second_survey_found_mixed_storm_and_wear_and_tear THEN cash_settlement_limited_to_storm_portion_is_fair; IF insurer_has_wear_and_tear_exclusion AND second_inspection_confirms_wear_and_tear_present THEN deduct_wear_and_tear_from_settlement; IF total_compensation_paid_is_adequate_for_delays_caused THEN no_additional_compensation_required</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3643634.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="120" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>STORM-018</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3819182</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Covea Insurance plc</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>9 Jan 2023</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Storm damage to roof during named storm November 2021 causing water ingress; Covea accepted storm conditions but declined citing pre-existing wear and tear highlighted by storm; agent inspection one month before the storm confirmed deterioration with slipped slates, silicon sealing and previous repairs; FOS gave more weight to pre-storm agent evidence than post-repair tradesman statements; internal and accidental damage claims also rejected</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Roof — slipped slates and deterioration with previous repairs confirmed by agent inspection one month before the storm in October 2021; two slates slipped and silicon used to seal slate; storm highlighted existing maintenance issues; internal water damage attributed to pre-existing gradual deterioration not storm</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>Covea's agent inspected the roof one month before the storm in October 2021 and reported signs of deterioration, slipped slates, silicon sealing and previous repairs; Covea concluded the storm highlighted pre-existing maintenance issues rather than being the dominant cause; internal damage also declined as resulting from gradual wear and tear; accidental damage rejected as wear and tear is excluded under the general exclusions</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Covea relied on its October 2021 pre-storm agent inspection report showing roof deterioration and slipped slates, and photos taken of the main roof from the front one month before the storm; Mrs B provided reports from a builder and roofer who both said damage was caused by storm not wear and tear; Mrs B argued Covea focused on the rear roof not the storm-damaged front; FOS gave more weight to the pre-storm photographic agent evidence than to post-repair tradesmen's opinions</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; Covea's decision confirmed as fair; agent's October 2021 inspection showing roof deterioration and slipped slates one month before the storm carried more weight than post-repair tradesmen's storm causation opinions; internal damage and accidental damage claims also rejected as wear and tear-driven; no award</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>Q3 answered no — a pre-storm agent inspection showing active deterioration (slipped slates, silicon sealing, previous repairs) one month before the storm carries more weight than post-repair tradesmen's opinions that the storm caused the damage; a storm that highlights or worsens existing maintenance issues is not the main cause of damage; accidental damage cover defined as unexpected physical damage by unidentifiable external means does not cover damage attributable to gradual wear and tear; the absence of further damage during subsequent storms does not prove the roof was in good condition before the first named storm</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>Evidence of roof condition at the storm-damaged front specifically, distinct from the October 2021 general inspection; independent expert assessment before repairs distinguishing storm-specific damage from the pre-existing deterioration; evidence contradicting the October 2021 agent report's findings on the main roof</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>Q1 — named storm conditions not disputed; Q2 — damage consistent with storm damage; Q3 — October 2021 agent inspection one month before storm found deterioration, slipped slates, silicon sealing and previous repairs; FOS gave this more weight than post-repair tradesmen's statements; storm highlighted existing maintenance issues; Mrs B's argument that Covea focused on rear roof not accepted as agent report covered the main roof from the front; no further damage in subsequent storms not determinative of pre-storm roof condition; accidental damage rejected — policy definition requires unexpected damage by unidentifiable external means, excluding wear and tear under general exclusions</t>
+        </is>
+      </c>
+      <c r="S19" s="5" t="inlineStr">
+        <is>
+          <t>A pre-storm agent inspection showing active deterioration (slipped slates, silicon sealing) is the most powerful Q3 evidence available — reference it specifically in decline reasoning; post-repair tradesmen's storm causation opinions carry less weight than pre-storm photographic inspections; accidental damage cover with a wear and tear exclusion does not provide a fallback route when storm damage fails on a wear and tear basis; the absence of further damage in subsequent storms does not prove the roof was in good condition before the first storm — repairs may have been effective</t>
+        </is>
+      </c>
+      <c r="T19" s="5" t="inlineStr">
+        <is>
+          <t>IF pre_storm_inspection_shows_active_deterioration_within_weeks_of_storm AND post_repair_tradesmen_say_storm_damage THEN pre_storm_inspection_carries_more_weight AND storm_q3 = no; IF storm_highlighted_existing_maintenance_issues_confirmed_by_pre_storm_report THEN storm_not_main_cause AND decline_reasonable; IF accidental_damage_cover_excludes_wear_and_tear AND damage_attributable_to_gradual_deterioration THEN accidental_damage_claim_also_fails</t>
+        </is>
+      </c>
+      <c r="U19" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3819182.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="120" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>STORM-019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3829618</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Royal &amp; Sun Alliance Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>19 Jan 2023</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Storm damage claim for water ingress to upstairs bedroom ceiling and kitchen; RSA's loss adjuster found no roof ingress and identified rotten window frames with visible daylight through holes as the main water source; ceiling damage described as pre-existing and not a one-off event; Mrs S could not provide evidence of prior roof repairs; Q2 failed on loss adjuster's identification of alternative non-storm ingress source</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Rotten window frames in upstairs bedroom with daylight visible through holes — RSA's loss adjuster identified these as the main ingress source not the roof; bedroom ceiling damage described as pre-existing bowing not consistent with one-off storm event; internal damage described as wear and tear with decayed timber; flat roof inspected and not flagged as a concern</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>RSA's loss adjuster found no water entering through the ceiling and identified rotten window frames with visible daylight through holes as the main ingress source; bedroom ceiling damage described as pre-existing and not a one-off event; internal damage described as wear and tear issues with decayed timber not consistent with storm damage; flat roof inspected and not flagged</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>RSA relied on loss adjuster's detailed assessment with photos identifying rotten windowsill as the main ingress source and describing internal damage as wear and tear with decayed timber; Mrs S argued water was entering through the roof not the windowsill and said the roof had been repaired previously; Mrs S could not provide evidence of prior roof repairs; Mrs S's own photos broadly showed the same findings as the survey report; FOS agreed the survey should be relied on as nothing contradicted it</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; RSA's decision confirmed as fair; loss adjuster's identification of rotten window frames as main ingress source not contradicted; ceiling damage pre-existing; internal damage consistent with gradual wear and tear not storm; Mrs S's unsubstantiated claim of prior roof repairs not determinative; no award</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P20" s="3" t="inlineStr">
+        <is>
+          <t>Q2 failed — where a loss adjuster identifies a specific non-storm source of ingress (rotten window frames with visible daylight) supported by photos and describes internal damage as pre-existing and wear and tear, the damage is not consistent with storm damage; a policyholder's assertion that water came from a different source requires corroborating evidence to displace the survey finding; unsubstantiated claims of prior roof repairs without evidence do not establish the roof as the ingress source; if the policyholder's own photographs show the same findings as the survey, the survey should be relied on</t>
+        </is>
+      </c>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>Evidence of prior roof repairs; photographs or independent expert assessment identifying the roof as the active ingress source; evidence distinguishing roof ingress from window frame ingress; evidence contradicting the loss adjuster's identification of rotten window frames as the main source</t>
+        </is>
+      </c>
+      <c r="R20" s="3" t="inlineStr">
+        <is>
+          <t>Q1 — storm conditions confirmed; Q2 — loss adjuster found no water entering through ceiling and identified rotten window frames with visible holes as main ingress; bedroom ceiling described as pre-existing bowing and not a one-off event; internal damage described as wear and tear with decayed timber; loss adjuster found water puddles on flat roof but attributed these to recent rainfall not active roof ingress; Q2 answered no; Mrs S's photos broadly showed same findings as survey; prior roof repair claim unsubstantiated; no evidence given to contradict survey; RSA's report relied on</t>
+        </is>
+      </c>
+      <c r="S20" s="3" t="inlineStr">
+        <is>
+          <t>When a loss adjuster identifies a specific alternative non-storm ingress source confirmed by photos, this defeats Q2; a policyholder who asserts a different ingress source but cannot provide corroborating evidence will not displace a survey supported by photos; post-claim photographs from the policyholder that show the same findings as the survey reinforce the insurer's position; prior repairs are a valid basis to support a storm claim only if evidenced — an unsubstantiated assertion of prior repairs does not establish the claimed ingress source</t>
+        </is>
+      </c>
+      <c r="T20" s="3" t="inlineStr">
+        <is>
+          <t>IF loss_adjuster_identifies_specific_non_storm_ingress_source AND confirmed_by_photos THEN storm_q2 = no AND decline_reasonable; IF policyholder_asserts_different_ingress_source AND cannot_provide_corroborating_evidence THEN policyholder_assertion_insufficient_to_displace_survey; IF internal_damage_described_as_pre_existing_and_wear_and_tear THEN storm_q2 = no; IF policyholder_photos_show_same_findings_as_survey THEN survey_evidence_reinforced</t>
+        </is>
+      </c>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3829618.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="120" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>STORM-020</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>DRN-4293834</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>17 Oct 2023</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Storm damage claim for gas flue chimney cowl blown off during winds of 5 January 2023; weather data showed peak winds of 43mph against policy threshold of 55mph (Storm Force 10); surveyor found cowl showed decay and material breakdown not storm damage; Q1 and Q3 both failed; accidental damage claim also failed as wear and tear excluded under that section</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Gas flue chimney cowl — surveyor found signs of decay to the grated section with breakdown in the material identified as the cause; remaining part of cowl still in chimney stack; weather data showed peak winds of 43mph below the 55mph policy storm definition</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>Weather data showed peak winds of 43mph below the policy storm threshold of 55mph (48 knots Storm Force 10); surveyor found the chimney cowl had signs of decay to the grated section with breakdown in the material identified as the cause; remaining part of cowl still in chimney stack; accidental damage section also excluded wear and tear</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>AXA relied on local weather data showing peak winds of 43mph and surveyor's report with clear photos showing decay and material breakdown; Mr D argued severe winds occurred overnight on 5 January 2023 and that aluminium does not rot or corrode; FOS noted aluminium can corrode and there was no evidence of equal weight to support Mr D's view; FOS agreed Q1 failed on weather data and Q3 failed on surveyor evidence</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; AXA's decision confirmed as fair; Q1 failed — weather data showed peak winds of 43mph below 55mph policy threshold; Q3 also failed — surveyor found material decay and breakdown as cause with photographic evidence; accidental damage claim also failed as wear and tear excluded under that section; no award</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P21" s="5" t="inlineStr">
+        <is>
+          <t>Q1 failed — where weather records show peak winds of 43mph against a policy threshold of 55mph (Storm Force 10), storm conditions are not met even if the policyholder believes severe winds occurred overnight; Q3 also failed — surveyor's clear photographic evidence of material decay is sufficient to establish a non-storm cause where the policyholder provides no evidence of equal weight; aluminium can corrode and an insurer is entitled to rely on photographic evidence of decay; wear and tear exclusion in the accidental damage section prevents the policyholder using that section as a fallback when storm damage is declined on wear and tear grounds</t>
+        </is>
+      </c>
+      <c r="Q21" s="5" t="inlineStr">
+        <is>
+          <t>Weather data showing winds meeting the 55mph policy threshold on 5 January 2023; independent expert assessment contradicting the surveyor's finding of material decay; evidence that the cowl was in good condition before the claim; evidence that the specific aluminium cowl had not corroded</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="inlineStr">
+        <is>
+          <t>Q1 — local weather data showed peak winds of 43mph; policy requires 55mph (48 knots Storm Force 10); storm conditions not met; Q1 answered no; Q2 — chimney cowl blowing off could be consistent with storm damage; Q3 — surveyor found decay to grated section and remaining part still in stack indicating material breakdown not physical dislodgement by wind; surveyor provided clear photos; Mr D's argument that aluminium does not corrode rejected as aluminium can corrode; no evidence of equal weight to support Mr D; Q1 and Q3 both no; accidental damage also declined as wear and tear exclusion applies to that section</t>
+        </is>
+      </c>
+      <c r="S21" s="5" t="inlineStr">
+        <is>
+          <t>Q1 failure on weather records alone defeats a storm claim — where local weather data clearly shows peak winds below the policy threshold, proceed no further; always check accidental damage section exclusions before suggesting it as a fallback for declined storm claims — wear and tear exclusions often apply there too; a surveyor's photographic evidence of material decay defeats Q3 unless the policyholder produces evidence of equal weight; a policyholder's belief that winds were severe is insufficient to override recorded weather data showing sub-threshold winds</t>
+        </is>
+      </c>
+      <c r="T21" s="5" t="inlineStr">
+        <is>
+          <t>IF local_weather_data_shows_peak_winds_below_policy_storm_threshold THEN storm_q1 = no AND claim_fails; IF surveyor_finds_material_decay_with_photographic_evidence AND policyholder_provides_no_evidence_of_equal_weight THEN storm_q3 = no AND decline_reasonable; IF storm_damage_declined_and_policyholder_seeks_accidental_damage AND accidental_damage_section_excludes_wear_and_tear AND damage_is_material_decay THEN accidental_damage_claim_also_fails</t>
+        </is>
+      </c>
+      <c r="U21" s="4" t="inlineStr">
+        <is>
+          <t>DRN-4293834.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add STORM-021 to STORM-025 to Storm Case Database
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Storm_Case_Database.xlsx
+++ b/knowledge/case-databases/Storm_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:U26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2703,6 +2703,531 @@
         </is>
       </c>
     </row>
+    <row r="22" ht="120" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>STORM-021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4517146</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>AXA XL Insurance Company UK Limited</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>23 Apr 2024</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Storm damage to balcony tiles on residential property partially declined; insurer paid internal damage but declined external tile replacement and scaffolding costs on grounds of wear and tear and sub-storm wind speeds</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Tiles lifted from balcony (one year old) allowing rainwater ingress into building interior; property in exposed position but no corroborating evidence of locally enhanced wind speeds</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Partial</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Weather records showed wind speeds insufficient for storm conditions; expert surveyor report cited wear and tear rather than storm damage with photos from the balcony and exterior; scaffolding cost excluded as consequential to declined external repair</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>AXA: weather records showing no storm-level winds, expert surveyor report citing wear and tear with balcony and exterior photographs. Policyholders: one-year-old tiles should not have failed without storm force, property in exposed position with argued higher localised winds, logical wind/rain causation — conceded balcony floor wear and tear but disputed tile damage</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; AXA's decision upheld as fair and in line with policy terms; tile damage and scaffolding decline confirmed; internal damage settlement not disturbed</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P22" s="3" t="inlineStr">
+        <is>
+          <t>Storm peril requires violent winds; burden of proof on policyholder to evidence storm conditions; an unsubstantiated claim of enhanced localised wind speeds due to exposed position requires corroborating evidence; insurer entitled to rely on expert surveyor report where report includes on-site photographs; scaffolding costs excluded where the underlying external repair is itself not storm-caused</t>
+        </is>
+      </c>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>Corroborating evidence of enhanced wind speeds at the exposed property location; independent expert assessment showing tile damage pattern inconsistent with wear and tear</t>
+        </is>
+      </c>
+      <c r="R22" s="3" t="inlineStr">
+        <is>
+          <t>Weather records for the period did not indicate storm-level wind speeds; policyholders could not provide corroborating evidence that localised conditions were more severe than nearby stations; AXA's expert report included balcony and exterior photos so could not be dismissed as inadequate; scaffolding was needed solely for the declined external repairs and therefore also excluded; policyholders themselves accepted the balcony floor wear and tear exclusion</t>
+        </is>
+      </c>
+      <c r="S22" s="3" t="inlineStr">
+        <is>
+          <t>An unsubstantiated exposed-position argument for enhanced localised winds is insufficient to establish storm conditions where weather records show sub-storm speeds; where the insurer's expert obtains photographs from the actual claimed damage location, the report cannot be challenged as inadequate; scaffolding costs follow the fate of the underlying repair — if the external damage is excluded, so is the access cost</t>
+        </is>
+      </c>
+      <c r="T22" s="3" t="inlineStr">
+        <is>
+          <t>IF weather_records_show_no_storm AND policyholder_claims_enhanced_local_winds AND no_corroborating_evidence THEN storm_q1 = no AND claim_fails; IF external_damage_declined_as_non_storm THEN consequential_scaffolding_cost_also_declined; IF insurer_expert_report_includes_on_site_photographs THEN report_cannot_be_dismissed_as_inadequate</t>
+        </is>
+      </c>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4517146.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="120" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>STORM-022</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>DRN-4757581</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Accredited Insurance (Europe) Ltd</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>4 Jul 2024</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Storm damage claim for water ingress through roof declined; insurer found no storm conditions and pre-existing wear and tear from failed previous repairs; claimant subsequently alleged cricket ball impact as alternative cause; both primary and alternative causes rejected</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Roof tiles previously repaired with subsequently failed repairs; broken tiles allowed rainwater to enter roof void; no storm conditions in weeks prior to damage being reported</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>No storm conditions confirmed in weeks prior to damage; approved surveyor found broken tiles with previously failed prior repairs constituting wear and tear and poor workmanship; cricket ball impact claimed as alternative but unsupported by evidence; gradual damage excluded under policy clause 12 and accidental damage cover not included in policy</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>Accredited: weather data confirming no storm conditions, approved surveyor report finding previously repaired tiles with failed repairs. Claimant: initially reported storm damage as he was not a roof expert; after seeing surveyor images alleged cricket ball impact from nearby cricket club; said damage happened over time causing ceiling collapse; no evidence provided for either cause</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; Accredited's decline on storm and wear and tear grounds confirmed; cricket ball alternative also rejected as unsupported by evidence and in any event caught by gradual damage exclusion and absence of accidental damage cover</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P23" s="5" t="inlineStr">
+        <is>
+          <t>Storm Q1 failed — no storm conditions in weeks prior to damage; policy general exclusion clause 12: 'Any gradual or maintenance-related loss or damage' including wear and tear and gradual deterioration whether aware or not; accidental damage cover not included in policy; for a claim to succeed the damage must be caused by an insured peril — no insured peril established under any head</t>
+        </is>
+      </c>
+      <c r="Q23" s="5" t="inlineStr">
+        <is>
+          <t>Evidence of storm conditions in the relevant period; evidence of cricket ball impact; evidence of a sudden damage event; evidence of roof condition immediately before the damage</t>
+        </is>
+      </c>
+      <c r="R23" s="5" t="inlineStr">
+        <is>
+          <t>Weather data and Accredited's evidence both confirmed no storm conditions; surveyor found pre-existing tiles with failed prior repairs; cricket ball alternative unsupported by evidence and even if proven would be gradual damage excluded under clause 12; accidental damage cover not in the policy; no insured peril established under any argument advanced</t>
+        </is>
+      </c>
+      <c r="S23" s="5" t="inlineStr">
+        <is>
+          <t>Where a claimant switches claimed peril after initial decline, assess each alternative independently — switching does not reset the burden of proof; a gradual damage exclusion can defeat both the primary storm claim and any subsequent alternative cause if both involve gradual deterioration; confirm whether accidental damage cover is included in the policy before it can be considered as a fallback</t>
+        </is>
+      </c>
+      <c r="T23" s="5" t="inlineStr">
+        <is>
+          <t>IF no_storm_conditions AND surveyor_finds_pre_existing_failed_repairs THEN decline_storm_and_wear_and_tear; IF alternative_cause_claimed_post_decline AND alternative_cause_also_gradual AND gradual_damage_excluded THEN alternative_cause_also_fails; IF no_accidental_damage_cover_in_policy THEN accidental_damage_fallback_unavailable</t>
+        </is>
+      </c>
+      <c r="U23" s="4" t="inlineStr">
+        <is>
+          <t>DRN-4757581.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="120" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>STORM-023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4899211</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>U K Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>23 Aug 2024</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Storm damage claim for water ingress from roof and guttering overflow declined; insurer found no storm conditions and attributed cause to guttering maintenance or defect; internal damage separately covered under accidental damage section; service failures acknowledged with £200 compensation</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Guttering overflow from volume of rainfall allowing water to seep through leadwork at roof edges; no tiles displaced or structurally damaged; battens and felt replacement attributed to maintenance issue or defective guttering system</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Partial</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Local weather station data showed no storm conditions on or around the date of loss; surveyor found no evidence of storm damage — no displaced tiles; guttering overflow from rain volume attributed to maintenance issue or possible defective guttering; battens and felt replacement deemed maintenance; internal damage covered separately under accidental damage section</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>Insurer: local weather station data, surveyor report finding no storm damage and guttering overflow mechanism. Claimants: Met Office weather warning covering a large geographic area; challenged surveyor conduct; alleged claim mixed up with unrelated claim by agent; felt coerced into low initial internal cash settlement (later increased after second visit)</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold storm claim; decline confirmed; internal damage under accidental damage section not disturbed; UKI's £200 compensation for service failures endorsed as fair and proportionate; no further action required</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P24" s="3" t="inlineStr">
+        <is>
+          <t>Storm defined as violent winds accompanied by heavy rainfall or snow (ABI definition); geographically broad Met Office weather warning is insufficient to establish localised storm conditions at a specific property — local weather station data takes precedence; guttering overflow from rain volume is a maintenance or defective system issue not storm damage; storm and accidental damage sections are independent — external storm claim can be declined while internal accidental damage is accepted under a separate section</t>
+        </is>
+      </c>
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>Specific local weather data for the claimants' property showing storm-level wind speeds; evidence of displaced tiles or structural storm damage rather than guttering overflow mechanism</t>
+        </is>
+      </c>
+      <c r="R24" s="3" t="inlineStr">
+        <is>
+          <t>Weather station data for nearest stations showed no storm conditions; Met Office warning covered a wide area and was not specific to claimants' location; no tiles displaced or damaged — guttering backed up allowing water through leadwork, consistent with maintenance or defect not storm; UKI applied separate sections correctly — internal damage was sudden and unintentional so covered under accidental damage; service failures (mixed-up claim, low initial offer, coercion) real but £200 already offered by UKI endorsed as proportionate</t>
+        </is>
+      </c>
+      <c r="S24" s="3" t="inlineStr">
+        <is>
+          <t>A broad regional weather warning does not substitute for local weather station data showing storm-level winds at the specific property; guttering overflow from heavy rain is not storm damage even when rain accompanies otherwise stormy weather; declining storm damage while accepting internal accidental damage under a separate policy section is independently valid; when service failures are acknowledged and compensated before FOS, the FOS-endorsed figure sets the ceiling unless further harm is shown</t>
+        </is>
+      </c>
+      <c r="T24" s="3" t="inlineStr">
+        <is>
+          <t>IF weather_warning_covers_large_area AND local_station_shows_no_storm THEN storm_conditions_not_established; IF damage_mechanism_is_guttering_overflow AND no_tiles_displaced THEN storm_q2 = no AND classify_as_maintenance_or_defect; IF storm_section_declined AND accidental_damage_section_applies_independently THEN internal_damage_may_still_be_covered_under_ad_section</t>
+        </is>
+      </c>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4899211.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="120" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>STORM-024</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5647934</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>AXIS Specialty Europe SE</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>18 Jan 2026</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Storm damage claim for boundary fence blown down declined; insurer applied explicit policy exclusion for storm damage to fences under the storm, flood or weight of snow peril despite fences being within the policy definition of buildings</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Boundary fence blown down by storm; no water ingress — structural storm damage to garden boundary structure only</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>Policy booklet right-hand 'What is not covered' column alongside the storm peril explicitly excludes 'loss or damage to... gates and fences'; exclusion wording clear and unambiguous; storm conditions and fence damage not disputed; the buildings definition including fences does not override the storm-peril-specific fence exclusion</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>Insurer: policy booklet exclusion column c) under storm peril explicitly naming fences; FOS confirmed wording unambiguous. Claimant: fences within buildings definition, storm definition met (&gt;47mph), argued exclusion wording was ambiguous, referenced Clause 4 Storm Exclusion Clause as most relevant text — however Clause 4 was not listed in the policy schedule and therefore inapplicable</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; AXIS's decline confirmed as fair; storm-peril exclusion for fences is clear and unambiguous; Clause 4 endorsement not listed in policy schedule so inapplicable to this policy; no award</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P25" s="5" t="inlineStr">
+        <is>
+          <t>A specific peril-level exclusion for fences listed in the storm section 'What is not covered' column overrides the general buildings definition that includes fences; fences within the buildings definition does not mean storm damage to fences is covered; only endorsements listed in the policy schedule apply to that policy — a clause printed in the booklet but absent from the schedule is inapplicable; storm damage to fences is a standard industry exclusion and need not also appear in the general exclusions section</t>
+        </is>
+      </c>
+      <c r="Q25" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable — purely a policy wording dispute; no factual evidence gaps</t>
+        </is>
+      </c>
+      <c r="R25" s="5" t="inlineStr">
+        <is>
+          <t>Storm conditions and fence damage not in dispute; policy booklet used a box format with 'What is covered' left and 'What is not covered' right; right-hand column alongside storm peril listed three specific exclusions including 'gates and fences'; this is separate from and overrides the general buildings definition; Clause 4 in the booklet headed 'Storm Exclusion Clause' not listed in the policy schedule as an applicable endorsement and therefore does not apply; Mrs R's ambiguity arguments rejected — three exclusions in the right-hand column are separate items each read independently</t>
+        </is>
+      </c>
+      <c r="S25" s="5" t="inlineStr">
+        <is>
+          <t>Check both the storm peril's own exclusion column and the general exclusions separately — a specific peril-level exclusion for fences is valid regardless of the buildings definition; verify which endorsements are listed in the policy schedule before applying or arguing a booklet clause; explicitly cite the exact policy wording of the fence exclusion in decline letters to pre-empt ambiguity arguments</t>
+        </is>
+      </c>
+      <c r="T25" s="5" t="inlineStr">
+        <is>
+          <t>IF claimed_item IN ['fence', 'gate'] AND policy_storm_peril_exclusion_includes_fences THEN decline_storm_claim_regardless_of_buildings_definition; IF endorsement_in_booklet AND endorsement_not_listed_in_policy_schedule THEN endorsement_inapplicable; IF buildings_definition_includes_item AND storm_peril_exclusion_also_names_item THEN storm_peril_exclusion_prevails</t>
+        </is>
+      </c>
+      <c r="U25" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5647934.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="120" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>STORM-025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>DRN-6075693</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>20 Feb 2026</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Storm damage claim for structural damage to flat (wall head gutter and cornice) declined by current insurer AXA; damage established by prior Ombudsman decision and structural engineer report as gradual and cumulative from successive storms in 2021-2022, predating AXA policy start date of 31 December 2022</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Wall head gutter and cornice — cumulative structural deterioration from successive storms from 2021 onwards; storms progressively loosened masonry bond allowing water penetration and further accelerated deterioration; damage gradual not sudden</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Leasehold flat</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Inception Damage Dispute</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>AXA policy incepted 31 December 2022; prior Ombudsman final decision and chartered structural engineer report established damage was gradual and cumulative from successive storms in 2021-2022, all predating AXA's policy period; AXA not required to respond to claims for events occurring before it was on risk; claimant's discovery of the cause in January 2023 does not shift liability to AXA</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>AXA: prior Ombudsman final decision against previous insurer F; chartered structural engineer report (D) describing 'cumulative effects of damage from successive storms' from 2021 with progressive masonry loosening; claimant's own statements referencing November 2022 storm and January 2023 catastrophic collapse. Claimant: argued damage could have occurred due to a storm in January 2023 within AXA's policy period; disputed the gradual nature; said he did not know he had cause to claim until January 2023</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; AXA's decline confirmed as fair; prior Ombudsman decision and structural engineer report established damage predated AXA policy period; claimant's ignorance of the cause is irrelevant to which insurer is on risk; no award</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P26" s="3" t="inlineStr">
+        <is>
+          <t>Insurer on risk not required to consider claims for events occurring before its policy period started; storm cover requires sudden not gradual damage; cumulative effects of damage from successive storms over multiple years is gradual damage not a sudden storm event; policyholder's first awareness of the cause does not determine which insurer is liable; a prior Ombudsman final decision establishing the damage chronology is highly persuasive in subsequent related complaints</t>
+        </is>
+      </c>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>Evidence of a distinct sudden storm damaging event within AXA's policy period after 31 December 2022; evidence contradicting the structural engineer's finding of cumulative gradual damage commencing in 2021</t>
+        </is>
+      </c>
+      <c r="R26" s="3" t="inlineStr">
+        <is>
+          <t>Prior Ombudsman established damage was gradual from 2021 storms under previous insurer F; chartered structural engineer D described 'cumulative effects of damage from successive storms' in 2022 with progressive masonry loosening — not a sudden event; claimant's own statements in earlier complaints attributed damage to November 2022 storm predating AXA's cover; AXA policy only covers events after 31 December 2022; policyholder's ignorance of the cause does not shift risk to AXA; no evidence of a new distinct storm damaging event within AXA's period</t>
+        </is>
+      </c>
+      <c r="S26" s="3" t="inlineStr">
+        <is>
+          <t>Where a prior Ombudsman decision establishes the damage chronology for the same property damage, it is highly persuasive in subsequent related complaints and binds the factual finding; when consecutive policies are in play and damage is cumulative, liability rests with the insurer on risk when the damage originated — not when it became apparent to the policyholder; first-awareness date is irrelevant to which insurer is on risk; cumulative successive-storm damage is not a sudden storm event and falls outside the storm peril</t>
+        </is>
+      </c>
+      <c r="T26" s="3" t="inlineStr">
+        <is>
+          <t>IF damage_cause_predates_current_insurer_policy_start_date THEN current_insurer_not_liable REGARDLESS_OF_DISCOVERY_DATE; IF prior_ombudsman_decision_establishes_gradual_damage_and_pre_inception THEN current_insurer_may_rely_on_that_finding; IF damage_is_cumulative_successive_storms AND commenced_before_policy_inception THEN storm_peril_not_triggered_under_current_policy</t>
+        </is>
+      </c>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>DRN-6075693.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add STORM-026 to STORM-030 to Storm Case Database
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Storm_Case_Database.xlsx
+++ b/knowledge/case-databases/Storm_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U26"/>
+  <dimension ref="A1:U31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3228,6 +3228,531 @@
         </is>
       </c>
     </row>
+    <row r="27" ht="120" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>STORM-026</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>DRN0445901</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Gresham Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>30 Nov 2015</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Storm damage to exterior of residential home declined; water leaking into two bedrooms and living room in October 2014; two loss adjusters found wear and tear not storm damage; policyholders' roofer addressed damage scope only, not causation; internal repairs separately paid under accidental damage cover</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Roof — water ingress through roof covering to two bedrooms and living room; two loss adjusters found no storm damage; policyholders' roofer had better roof access but report addressed repair scope not storm causation</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Partial</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>Two independent loss adjusters both concluded damage was due to wear and tear not storm damage; one explicitly stated 'no storm damage to roof'; policyholders' own roofer's report addressed only the extent of damage and repair costs, not the cause of damage</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>Insurer: two concordant loss adjuster reports both finding wear and tear not storm damage, one explicitly stating no storm damage to roof; photographs reviewed. Policyholders: specialist roofer who accessed the roof directly and provided a repair quote; argued roofer's on-roof inspection was more thorough than loss adjusters' ground-level assessments; FOS accepted roofer had better access but found report silent on causation</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; Gresham's external damage decline confirmed as fair; Q2 failed — two concordant expert opinions of no storm damage not displaced by roofer's report which addressed repair scope only; internal repairs and £100 compensation already paid by Gresham pre-FOS not disturbed</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P27" s="5" t="inlineStr">
+        <is>
+          <t>Q2 failed — a policyholders' specialist report that addresses damage extent and repair costs but not storm causation carries no evidential weight on the Q2 question, even if the specialist had superior roof access; two concordant independent expert findings of no storm damage are sufficient to decline the storm peril even where the policyholder's expert had better physical access to the damage</t>
+        </is>
+      </c>
+      <c r="Q27" s="5" t="inlineStr">
+        <is>
+          <t>Expert opinion from policyholders' roofer specifically addressing storm causation (the report addressed repair scope only, not whether the damage was caused by a storm); independent assessment contradicting the two loss adjusters' concordant finding of no storm damage</t>
+        </is>
+      </c>
+      <c r="R27" s="5" t="inlineStr">
+        <is>
+          <t>Q1 — storms confirmed in the area in the ten days before the damage was reported; Q2 — two loss adjusters both found wear and tear not storm damage; one explicitly stated 'no storm damage to roof'; policyholders' roofer had better access to some roof areas but his report said nothing about the cause of damage — only what damage existed and the repair cost; FOS could not find anything in the roofer's report contradicting the two expert opinions; Q2 answered no; Q3 not considered</t>
+        </is>
+      </c>
+      <c r="S27" s="5" t="inlineStr">
+        <is>
+          <t>Two concordant loss adjuster reports finding no storm damage are sufficient to decline Q2 where the policyholder's counter-evidence (a roofer's report) is silent on causation; always ensure decline reasoning explicitly references the lack of causation opinion in the policyholder's counter-report — the report's silence on causation, not its access limitations, is the decisive point; internal accidental damage cover should be assessed independently from the storm peril at first handling to avoid separate complaint exposure</t>
+        </is>
+      </c>
+      <c r="T27" s="5" t="inlineStr">
+        <is>
+          <t>IF two_independent_expert_reports_find_no_storm_damage AND policyholder_counter_report_silent_on_causation THEN storm_q2 = no AND decline_reasonable; IF policyholder_report_addresses_repair_scope_only_not_causation THEN report_carries_no_weight_on_storm_q2; IF internal_damage_payable_under_accidental_damage THEN assess_independently_from_storm_peril_at_first_handling</t>
+        </is>
+      </c>
+      <c r="U27" s="4" t="inlineStr">
+        <is>
+          <t>DRN0445901.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="120" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>STORM-027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>DRN1086734</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>U K Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>12 Sep 2016</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Storm damage to roof causing water ingress declined; external roof repair declined and internal damage paid; winds reached storm threshold on only two isolated occasions and heavy rain came days later not concurrent; loss adjuster found no storm damage; policyholders did not commission specialist storm damage report despite UKI inviting one</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Roof — rainwater ingress through roof covering; loss adjuster found no evidence of storm damage and attributed cause to general maintenance issues; no expert report identifying storm-specific damage provided by policyholders</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Partial</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>Winds reached borderline storm level on only two isolated occasions and were not concurrent with the very heavy rain that came days later; loss adjuster found no evidence of storm damage to the roof, attributing cause to general maintenance issues; policyholders did not provide a specialist roofer's report confirming storm damage despite UKI offering to reconsider on that basis</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>Insurer: loss adjuster report finding no storm damage and identifying maintenance as the cause; weather records showing borderline winds on only two occasions not concurrent with heavy rain. Policyholders: high-profile storm warnings for their area; argued UKI's loss adjuster was not professional; did not commission a specialist roofer's storm damage report despite UKI's invitation to do so</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; external roof decline confirmed; Q1 borderline and unlikely to have damaged a well-maintained roof; Q2 failed — no expert evidence of storm damage to roof available; UKI's offer to reconsider on receipt of specialist report confirmed as fair and sufficient; no further action required</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P28" s="3" t="inlineStr">
+        <is>
+          <t>Where wind speeds are borderline and reached storm threshold on only isolated occasions without being concurrent with heavy rain, and the only professional evidence available is the loss adjuster's finding of no storm damage, the claim fails; an insurer's conditional offer to reconsider upon receipt of a specialist storm damage report is a fair and proportionate response that FOS will not improve upon; a policyholder who fails to commission an expert report when explicitly invited to do so cannot argue the insurer has not considered their position</t>
+        </is>
+      </c>
+      <c r="Q28" s="3" t="inlineStr">
+        <is>
+          <t>Specialist roofer's report confirming storm-specific damage to the roof (UKI offered to reconsider on this basis but no such report was provided)</t>
+        </is>
+      </c>
+      <c r="R28" s="3" t="inlineStr">
+        <is>
+          <t>Q1 — weather evidence showed consistently strong winds with storm-level gusts on only two isolated occasions; heavy rain came a few days later, not concurrent with the storm winds; FOS thought winds at this level unlikely to have damaged a well-maintained roof; Q2 — loss adjuster report found no evidence of storm damage, attributing cause to maintenance; policyholders provided no expert report contradicting this despite UKI's invitation; Q2 failed; UKI's offer to reconsider on receipt of specialist report confirmed as reasonable</t>
+        </is>
+      </c>
+      <c r="S28" s="3" t="inlineStr">
+        <is>
+          <t>Where winds are borderline and not concurrent with heavy rain, and the loss adjuster finds maintenance issues rather than storm damage, decline the storm peril and offer in writing to reconsider on receipt of a specialist storm damage report — this creates a fair and FOS-endorsed position; a policyholder who fails to take up that offer cannot subsequently argue the insurer made an uninvestigated decision</t>
+        </is>
+      </c>
+      <c r="T28" s="3" t="inlineStr">
+        <is>
+          <t>IF winds_borderline_storm_threshold AND not_concurrent_with_heavy_rain AND loss_adjuster_finds_no_storm_damage THEN storm_q1_and_q2_fail AND decline_reasonable; IF insurer_offers_to_reconsider_on_specialist_report AND policyholder_does_not_provide_report THEN insurer_position_confirmed_as_fair; IF no_expert_evidence_of_storm_damage_available THEN storm_q2 = no</t>
+        </is>
+      </c>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
+          <t>DRN1086734.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="120" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>STORM-028</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>DRN1681509</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Kwik-Fit Insurance Services Ltd</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>22 Jul 2016</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Home insurance policy mis-sold without storm cover despite being told it was included; broker accepted mis-selling and offered £100 compensation; FOS assessed whether storm claim would have succeeded if correct policy held — concluded no, as photos showed no storm damage and damage consistent with gradual deterioration</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Roof — water ingress attributed to gradual deterioration; loss adjuster found no missing tiles or blown-off felt; photos showed no evidence of storm damage; internal damage appeared to have occurred over a long period</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>Policy did not include storm cover (mis-sold); on hypothetical assessment, storm claim would have failed anyway — loss adjuster found no storm damage externally; photos showed no missing tiles or blown felt; internal damage appeared to have occurred over a long period; damage consistent with gradual deterioration over time not a storm event</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>Broker/insurer: loss adjuster report finding no storm damage; photographic evidence showing no missing tiles or blown-off felt. Claimant: builder's statement that roof was storm damaged and felt had been blown off; surveyor's letter confirming repair quotation was proportionate and fair (but not confirming storm causation); FOS found photos contradicted builder's storm claim and surveyor's letter addressed only cost proportionality not causation</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M29" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; Mr D no worse off from mis-selling — storm claim would have failed on the merits; £100 compensation already paid by Kwik-Fit for mis-selling adequate; no further action required</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" s="4" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P29" s="5" t="inlineStr">
+        <is>
+          <t>Where a policy is mis-sold, FOS assesses whether the policyholder is worse off by hypothetically evaluating whether the correct claim would have succeeded; photos showing no missing tiles, no blown-off felt, and internal damage consistent with long-term water ingress defeat Q2 and Q3; a builder's statement of storm damage and a surveyor's letter confirming only cost proportionality do not constitute expert storm causation evidence sufficient to displace loss adjuster photographic findings</t>
+        </is>
+      </c>
+      <c r="Q29" s="5" t="inlineStr">
+        <is>
+          <t>Expert storm causation opinion confirming the roof was damaged by a specific storm event (builder's statement and surveyor's cost letter did not address causation); photographs showing storm-consistent damage such as missing tiles or blown felt</t>
+        </is>
+      </c>
+      <c r="R29" s="5" t="inlineStr">
+        <is>
+          <t>Kwik-Fit accepted mis-selling; FOS assessed hypothetically whether storm claim would have succeeded if correct policy held; loss adjuster photos showed no missing tiles or blown-off felt; internal damage appeared to have occurred over a long period; on balance photos supported gradual deterioration not storm damage; builder's storm assertion not supported by photos; surveyor's letter confirmed only cost proportionality not storm causation; storm claim would most likely have failed; Mr D no worse off; £100 compensation adequate</t>
+        </is>
+      </c>
+      <c r="S29" s="5" t="inlineStr">
+        <is>
+          <t>When assessing mis-selling complaints involving storm claims, apply the same three-question framework hypothetically — if the underlying claim would have failed, the policyholder has not been materially harmed; photographic evidence of no missing tiles and no blown-off felt is sufficient to defeat Q2 where the policyholder's only counter-evidence is a builder's assertion and a cost-proportionality letter</t>
+        </is>
+      </c>
+      <c r="T29" s="5" t="inlineStr">
+        <is>
+          <t>IF policy_mis_sold AND storm_claim_would_fail_on_merits_hypothetically THEN policyholder_not_materially_worse_off AND compensation_for_mis_selling_only; IF photos_show_no_missing_tiles AND no_blown_felt AND internal_damage_gradual THEN storm_q2_and_q3 = no; IF counter_evidence_is_builder_assertion_and_cost_letter_only THEN insufficient_to_displace_photographic_loss_adjuster_findings</t>
+        </is>
+      </c>
+      <c r="U29" s="4" t="inlineStr">
+        <is>
+          <t>DRN1681509.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="120" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>STORM-029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>DRN2201217</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Elite Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>8 Jul 2018</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Storm damage to roof and internal damage declined in full; policy defined storm as Force 10 (55-63mph); maximum wind speed in month before claim was 40mph; surveyor found roof in poor condition due to age with loose nails and gaps; internal damage also declined as not accidental — water had leaked gradually over a period of time</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Roof — surveyor found poor condition due to age, with fixing nails working loose leaving gaps for water ingress; water leaked through to extension and kitchen ceiling over a period of time; no storm-force winds recorded</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>Policy defined storm as Force 10 winds of 55-63mph or above; weather records showed maximum wind speed of 40mph in the month before the claim — well below the policy threshold; surveyor found roof in poor condition due to age with loose nails creating gaps; internal damage also declined as not accidental — policy required damage to be sudden, unexpected, happening at a specific time, and caused by something external and identifiable; water had leaked over a period of time satisfying none of these conditions</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>Insurer: weather records showing maximum 40mph winds; surveyor report describing poor roof condition due to age with loose nails and gaps. Claimant: denied roof was in poor condition; had previously carried out some repairs; FOS accepted it was reasonable to rely on the expert surveyor evidence</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; both storm and accidental damage claims failed; Q1 failed on weather records (40mph against 55-63mph threshold); roof condition confirmed poor by surveyor; internal damage also excluded as water leaked gradually over time — not sudden, unexpected, or happening at a specific time as required by the accidental damage definition; no award</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P30" s="3" t="inlineStr">
+        <is>
+          <t>Policy-defined storm threshold of Force 10 (55-63mph); recorded maximum winds of 40mph clearly fail Q1 on numerical grounds; the accidental damage policy definition requiring damage to be 'sudden, unexpected, happening at a specific time, caused by something external and identifiable' excludes water ingress that has leaked gradually over a period of time — all four conditions must be met; prior repairs by a claimant do not displace a surveyor's contemporaneous finding of poor roof condition</t>
+        </is>
+      </c>
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>Weather data showing winds meeting the Force 10 / 55-63mph policy threshold; independent expert assessment contradicting the surveyor's finding of poor roof condition; evidence that water ingress was sudden and occurred at a specific identifiable time</t>
+        </is>
+      </c>
+      <c r="R30" s="3" t="inlineStr">
+        <is>
+          <t>Q1 — policy defines storm as Force 10 (55-63mph); weather records showed maximum 40mph in the month before the claim; 40mph is nowhere near sufficient to damage a roof in sound condition; Q1 answered no; surveyor found roof in poor condition due to age with loose fixing nails creating gaps; Ms D's prior repairs noted but expert evidence relied on; internal accidental damage assessed separately — policy required sudden, unexpected, at a specific time, caused by something external and identifiable; surveyor noted water had leaked over a period of time to extension and kitchen ceiling; does not meet any of the suddenness conditions; both claims declined</t>
+        </is>
+      </c>
+      <c r="S30" s="3" t="inlineStr">
+        <is>
+          <t>Where a policy contains an explicit numeric storm threshold (Force 10 / 55mph), cite the exact recorded wind speed and the threshold in the decline reasoning — the numerical gap speaks for itself; always assess accidental damage independently from the storm claim and check whether the policy's suddenness conditions are met — gradual water ingress fails the accidental damage definition even where storm also fails</t>
+        </is>
+      </c>
+      <c r="T30" s="3" t="inlineStr">
+        <is>
+          <t>IF policy_storm_threshold_numeric AND recorded_winds_below_threshold THEN storm_q1 = no AND decline; IF accidental_damage_requires_sudden_unexpected_specific_time AND water_ingress_was_gradual_over_period THEN accidental_damage_also_fails; IF surveyor_finds_poor_roof_condition AND policyholder_denies_AND_cites_prior_repairs THEN surveyor_contemporaneous_finding_takes_precedence</t>
+        </is>
+      </c>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>DRN2201217.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="120" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>STORM-030</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>DRN2738252</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>U K Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>20 Jun 2020</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Attic leak and wind-damaged door after stormy weather; UKI assessed from photographs without physical survey; roof repair declined as damage consistent with gradual build-up not storm; door damage paid under accidental damage; policyholders argued physical survey should have been required</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Roof valley between two roof sections — photographs showed accumulated debris and removed tiles in a sheltered location; repairs required clearing the valley and replacing battens and felt, consistent with gradual maintenance build-up; no damage reported to more exposed roof areas</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Partial</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>Photographs showed damage in sheltered roof valley with accumulated debris characteristic of long-term collection, not storm impact; no damage to more exposed roof areas as would be expected from a storm; repair scope (clearing valley, replacing battens and felt) typical of gradual maintenance build-up not a one-off storm event; physical survey not required where photographs are sufficiently clear</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>Insurer: photographs from policyholders showing debris-filled valley, removed tiles in sheltered location, and repair scope typical of gradual build-up; storm conditions in prior two weeks accepted. Policyholders: argued UKI should have conducted a physical survey before declining; said damage was caused by the storm; UKI agreed door damage was accidental</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M31" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; Q2 and Q3 failed — valley location with accumulated debris, no damage to exposed areas, and repair scope all inconsistent with storm as the main cause; physical survey not required; door accidental damage payment not disturbed; no further action required</t>
+        </is>
+      </c>
+      <c r="N31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P31" s="5" t="inlineStr">
+        <is>
+          <t>Q2 failed — damage located in a sheltered roof valley with accumulated debris is not consistent with storm damage; where storm damage to one area would be expected to cause more extensive damage to more exposed areas and none is reported, this undermines the storm causation argument; Q3 failed — repair scope of clearing a valley and replacing battens and felt is characteristic of gradual maintenance build-up not a one-off storm event; a physical survey is not required where photographic evidence is sufficiently clear to assess the claim</t>
+        </is>
+      </c>
+      <c r="Q31" s="5" t="inlineStr">
+        <is>
+          <t>Expert assessment establishing storm as the specific cause of the valley damage; evidence of intact roof condition immediately before the storm; evidence of damage to more exposed roof areas consistent with storm impact</t>
+        </is>
+      </c>
+      <c r="R31" s="5" t="inlineStr">
+        <is>
+          <t>Q1 — storm conditions in the two weeks before the claim accepted by UKI; Q2 — photos showed damage in valley between two roofs, a sheltered location; debris visible consistent with long-term accumulation; no damage to more exposed areas reported, which would be expected if storm had caused the valley damage; if pre-repair photo, did not show typical storm damage; Q2 answered no; Q3 — repair description (clearing valley, replacing battens and felt) typical of gradual build-up not one-off storm; valley may require more frequent maintenance by design; Q3 answered no; physical survey not required — reasonably clear photos sufficient; door damage correctly paid under accidental damage</t>
+        </is>
+      </c>
+      <c r="S31" s="5" t="inlineStr">
+        <is>
+          <t>A sheltered location (roof valley) combined with accumulated debris and no storm damage to more exposed areas is a strong Q2 failure argument — document both points explicitly in decline reasoning; the repair scope (clearing a valley, replacing battens and felt) is a reliable Q3 indicator of gradual build-up rather than storm impact; an insurer can rely on clear photographs in lieu of a physical survey — this is FOS-endorsed and does not give rise to a complaint</t>
+        </is>
+      </c>
+      <c r="T31" s="5" t="inlineStr">
+        <is>
+          <t>IF damage_in_sheltered_location AND accumulated_debris_visible AND no_damage_to_exposed_areas THEN storm_q2 = no; IF repair_scope_includes_clearing_valley_and_replacing_battens_and_felt THEN storm_q3 = no_as_gradual_buildup; IF photographic_evidence_sufficiently_clear THEN physical_survey_not_required AND insurer_position_not_undermined</t>
+        </is>
+      </c>
+      <c r="U31" s="4" t="inlineStr">
+        <is>
+          <t>DRN2738252.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add STORM-031 to STORM-035 to Storm Case Database
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Storm_Case_Database.xlsx
+++ b/knowledge/case-databases/Storm_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:U36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3753,6 +3753,531 @@
         </is>
       </c>
     </row>
+    <row r="32" ht="120" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>STORM-031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>DRN3019884</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Royal &amp; Sun Alliance Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>26 Oct 2015</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Storm damage to roof of residential home declined; Mr and Mrs M claimed storm damage; two independent experts appointed by RSA found no storm damage — second expert found no missing or dislodged slates or tiles, lead flashing intact, and roof deteriorating over years; policyholders' contractor claimed storm damage but could not displace two concordant expert opinions; prejudice from delayed claim handling noted but not determinative</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Roof — two expert inspections found no missing or dislodged slates or tiles, all lead flashing in good repair; damage attributed to multi-year deterioration not a storm event; policyholders' contractor claimed storm damage but provided no independent expert support</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>Two independent experts appointed by RSA found damage inconsistent with storm damage; second expert explicitly found no signs of a one-off insurable event, no missing or dislodged slates or tiles, and confirmed the roof had been deteriorating for years; policyholders' contractor's opinion of storm damage not supported by independent expert findings</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>RSA: two concordant expert reports both finding no storm damage; first expert noted damage had occurred a long time before and RSA's position was prejudiced as damage worsened over time; second expert found no missing or dislodged slates or tiles, lead flashing in good repair, no signs of a one-off insured event, roof deteriorating for years. Policyholders: their contractor said storm damage; argued claim was made months earlier but no forms were sent by RSA; neighbour's claim was settled by their insurer; internal damage also raised but excluded from complaint at policyholders' request</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; RSA's decline confirmed as fair; Q2 and Q3 answered no; contractor's assertion of storm damage insufficient to displace two concordant expert findings; prejudice from delayed claim handling noted but not determinative as storm damage itself not established; no award</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P32" s="3" t="inlineStr">
+        <is>
+          <t>Q2 and Q3 failed — two concordant expert findings of no storm damage, including explicit finding of no signs of a one-off insurable event and documented multi-year roof deterioration, are sufficient to decline the claim; a policyholders' contractor's assertion of storm damage does not displace two independent expert opinions finding no storm damage; prejudice from delayed claim handling is relevant only if the underlying storm damage claim would have succeeded — where Q2 fails it does not need to be resolved</t>
+        </is>
+      </c>
+      <c r="Q32" s="3" t="inlineStr">
+        <is>
+          <t>Expert evidence supporting storm causation (policyholders had only their contractor's opinion, not an independent expert report); evidence that damage was the result of a one-off insured event rather than progressive deterioration</t>
+        </is>
+      </c>
+      <c r="R32" s="3" t="inlineStr">
+        <is>
+          <t>Q1 — storms occurred in the area (no specific date pinpointed but accepted generally on overall records). Q2 — policyholders' contractor said storm damage; two RSA experts disagreed; second expert found no missing or dislodged slates or tiles, lead flashing in good repair, no signs of a one-off insurable event, roof deteriorating for years; answer to Q2 no. Q3 not considered once Q2 failed. RSA acted reasonably. Prejudice from delayed claim noted but not determinative once storm damage not established. Neighbour's claim with different insurer irrelevant. Internal damage excluded from complaint by policyholders.</t>
+        </is>
+      </c>
+      <c r="S32" s="3" t="inlineStr">
+        <is>
+          <t>Two concordant expert findings of no storm damage are sufficient to decline Q2; a contractor's storm assertion does not displace two independent expert reports where both find no signs of a one-off insurable event; where the underlying storm damage claim fails at Q2, prejudice arguments (delayed forms, late inspection) need not be resolved; confirm at first handling whether internal damage is also claimed and assess it separately to avoid creating a separate complaint head</t>
+        </is>
+      </c>
+      <c r="T32" s="3" t="inlineStr">
+        <is>
+          <t>IF two_independent_experts_find_no_storm_damage AND no_missing_or_dislodged_slates AND roof_deteriorating_years THEN storm_q2 = no AND decline_reasonable; IF policyholder_counter_evidence_is_contractor_assertion_only THEN insufficient_to_displace_concordant_expert_findings; IF storm_q2_fails THEN delay_prejudice_argument_need_not_be_resolved</t>
+        </is>
+      </c>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
+          <t>DRN3019884.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="120" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>STORM-032</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>DRN5013915</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Ageas Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>12 Sep 2019</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Storm damage to flat roof of residential home declined; January 2019 claim; felt and boards reported ripped off during high winds; Ageas declined based on a self-imposed 55mph storm threshold not in policy terms; FOS rejected threshold but found Q3 failed — 9+ year old unmaintained flat roof with no pre-storm condition evidence</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Flat roof — felt and boards underneath reported ripped off during high winds; policyholders had contractors carry out permanent repairs before any inspection could be arranged; repair invoice listed work done but did not establish storm causation</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>Ageas declined on basis of self-imposed 55mph storm threshold (not in policy terms — rejected by FOS); actual Q3 failure confirmed by FOS: flat roof had been in place for over 9 years without maintenance, approaching end of typical 10-15 year lifespan; no pre-storm condition report; repair invoice listed repairs carried out but not that storm was the main cause; immediate permanent repairs prevented any inspection to validate storm causation</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>Insurer: weather records showing 48mph winds; self-imposed 55mph policy storm threshold (not in policy — FOS rejected); no inspection carried out as repairs completed before Ageas could inspect. Policyholders: Met Office postcode-level data showing 58mph (closer to property); reported felt and boards ripped off; repair invoice; acknowledged flat roof had been in place 9+ years without any maintenance</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; Ageas 55mph threshold rejected as absent from policy terms; Q1 accepted (48-58mph can cause structural damage = storm); Q2 accepted (felt and boards ripped off consistent with storm); Q3 failed — flat roof 9+ years without maintenance, no pre-storm condition evidence, repair invoice shows repairs not causation; storm not established as main cause; no award</t>
+        </is>
+      </c>
+      <c r="N33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P33" s="5" t="inlineStr">
+        <is>
+          <t>An insurer cannot apply a numeric storm threshold (here 55mph) that does not appear in the policy wording; Q3 — a flat roof in place for over 9 years without maintenance, approaching the end of its typical 10-15 year lifespan, with no evidence of good repair prior to the storm, fails Q3 as it is more likely that the weather highlighted pre-existing deterioration rather than caused the damage; a repair invoice listing work done does not establish storm causation; the burden of proof is on the policyholder to show storm was the main cause — absent pre-storm condition evidence this cannot be met</t>
+        </is>
+      </c>
+      <c r="Q33" s="5" t="inlineStr">
+        <is>
+          <t>Pre-storm condition report showing flat roof was in good repair; specialist storm causation report establishing that the 9+ year old unmaintained flat roof was damaged by the specific storm rather than pre-existing deterioration; expert inspection of damage (prevented by immediate permanent repairs)</t>
+        </is>
+      </c>
+      <c r="R33" s="5" t="inlineStr">
+        <is>
+          <t>Q1 — weather records showed minimum 48mph; Met Office postcode data showed 58mph; FOS accepted structural damage could arise at these speeds; Ageas 55mph threshold not in policy terms and potentially unfair; Q1 yes. Q2 — felt and boards ripped off is consistent with storm damage; Q2 yes. Q3 — onus on policyholders to show storm was main cause; flat roof in place 9+ years without any maintenance; flat roofs typically last 10-15 years; damage could have been storm-caused but more likely weather highlighted pre-existing issues; no pre-storm condition report; invoice lists repairs only not causation; immediate repairs prevented inspection; Q3 no.</t>
+        </is>
+      </c>
+      <c r="S33" s="5" t="inlineStr">
+        <is>
+          <t>A self-imposed policy storm threshold (55mph) not in policy wording will be rejected by FOS; where a flat roof is nearing the end of its typical lifespan with no maintenance history, Q3 is likely to fail unless the policyholder can evidence good pre-storm condition; document any spontaneous policyholder admissions about roof age and maintenance history at FNOL as these are key Q3 evidence; a repair invoice alone does not establish storm causation</t>
+        </is>
+      </c>
+      <c r="T33" s="5" t="inlineStr">
+        <is>
+          <t>IF insurer_storm_threshold_not_in_policy THEN threshold_cannot_be_applied AND q1_assessed_on_standard_structural_damage_criteria; IF flat_roof AND roof_age_approaching_end_of_lifespan AND no_maintenance_history AND no_pre_storm_condition_report THEN storm_q3 = no; IF repair_invoice_lists_repairs_only_not_causation THEN insufficient_to_establish_q3; IF immediate_repairs_prevent_inspection THEN does_not_relieve_policyholder_of_q3_burden</t>
+        </is>
+      </c>
+      <c r="U33" s="4" t="inlineStr">
+        <is>
+          <t>DRN5013915.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="120" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>STORM-033</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>DRN5397298</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>U K Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>28 Aug 2015</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Storm damage to garden wall of residential home; brick boundary wall with trellis collapsed; UKI declined on wear and tear grounds; loss adjuster report given reduced weight due to factual errors including wrong insurer and inapplicable exclusion cited; FOS found storm was most likely dominant cause and upheld the complaint</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Garden wall — boundary brick wall with small trellis on top blown over and collapsed in one piece; no roof water ingress; structural storm damage to boundary structure</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>UKI's surveyor found mould growth to mortar joints, nearby vegetation reducing structural strength, and no similar storm damage to surrounding fences facing the same direction; claim declined on wear and tear grounds</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>UKI: loss adjuster report citing mould growth to joints, nearby vegetation, and no similar damage to surrounding fences. Policyholders: no wear and tear exclusion in their policy (only a maintenance condition); photographs of wall before and after collapse; incurred telephone and postage costs chasing UKI for response over two months. FOS: reduced reliance on loss adjuster report due to factual errors — wrong insurer cited, wear and tear exclusion cited that did not exist in the policy</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>FOS upheld complaint; UKI required to: settle the storm claim for wall collapse with 8% simple interest on cash settlement; reimburse cost of replacement fence erected due to declined claim with 8% simple interest; pay £30.51 for telephone calls and postage costs; pay £100 compensation for distress and inconvenience</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P34" s="3" t="inlineStr">
+        <is>
+          <t>A loss adjuster's report carries reduced weight where it contains factual errors including citing the wrong insurer and applying a wear and tear exclusion that does not exist in the policy; photographs showing a wall fell in one piece and broke on impact are consistent with Q2 (blown over by storm-force wind); where there is no wear and tear exclusion in the policy (only a maintenance condition) the insurer cannot decline on that basis; neighbouring structures withstanding a storm is not conclusive against Q3 — shielding effects may explain the difference; a policyholder who cannot rebuild a declined structure is entitled to reimbursement of reasonable temporary remediation costs incurred as a direct consequence</t>
+        </is>
+      </c>
+      <c r="Q34" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — FOS found storm causation established on balance of photographic evidence and discredited loss adjuster report</t>
+        </is>
+      </c>
+      <c r="R34" s="3" t="inlineStr">
+        <is>
+          <t>Q1 not disputed — storm on the day confirmed. Q2 — photographs showed wall fell in one piece and broke on impact with ground, consistent with being blown over by storm-force wind; yes. Q3 — UKI's loss adjuster cited mould growth to mortar joints, vegetation, and unaffected neighbouring fences; FOS placed reduced reliance on this report due to errors (wrong insurer referenced, wear and tear exclusion cited that did not exist in the policy — policy had a maintenance condition instead); photographs of wall before and after showed only minor weathering and limited moss, not enough to cause collapse without storm; small vegetation across bottom not shown to grow into wall affecting structural integrity; neighbouring fences may have been shielded by the wall; on balance storm was most likely dominant cause and wall would probably have remained intact but for storm.</t>
+        </is>
+      </c>
+      <c r="S34" s="3" t="inlineStr">
+        <is>
+          <t>Accuracy of decline documentation is critical — a loss adjuster report citing the wrong insurer or an inapplicable exclusion will carry reduced weight at FOS; always verify the exact policy exclusions before issuing a decline and ensure the surveyor has checked the actual policy wording; where a policyholder incurs reasonable remediation costs as a direct consequence of a wrongly declined claim, reimbursement will be required; a neighbour's structure withstanding a storm is not conclusive — consider shielding effects before relying on this as Q3 evidence</t>
+        </is>
+      </c>
+      <c r="T34" s="3" t="inlineStr">
+        <is>
+          <t>IF loss_adjuster_report_contains_factual_errors_including_wrong_exclusion_cited THEN report_weight_reduced; IF wall_fell_in_one_piece_and_broke_on_impact THEN storm_q2 = yes; IF no_wear_and_tear_exclusion_in_policy THEN cannot_decline_on_wear_and_tear_grounds; IF policyholder_incurs_reasonable_remediation_costs_due_to_wrongly_declined_claim THEN reimbursement_required</t>
+        </is>
+      </c>
+      <c r="U34" s="2" t="inlineStr">
+        <is>
+          <t>DRN5397298.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="120" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>STORM-034</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>DRN7021460</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Liverpool Victoria Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>21 Jul 2017</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Storm damage to roof of residential home in exposed location; LV paid initial £5,000 for 2016 storm damage but declined additional £21,000 quote; policyholder had history of multiple prior claims (2012-2015) and could not produce invoices proving prior settled repairs were carried out; LV inspector also found non-storm causes</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Roof — LV inspector found some storm damage but also inferior valley lead, tile damage consistent with workmanship not storm, and crumbling ridge mortar from gradual deterioration; policyholder's roofer reported sagging from water ingress following storm tile dislodgement; engineer's report addressed structural integrity only, not specific leaking areas or repair scope</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Partial</t>
+        </is>
+      </c>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
+          <t>Policyholder could not provide invoices showing prior settled claims (2013, 2014, 2015) had been paid for and repairs carried out; LV inspector found non-storm causes including workman damage to tiles, inferior valley lead quality, and crumbling ridge mortar; engineer's report established general structural soundness but did not identify which areas were leaking, how long problems had existed, or what repairs were needed for the specific disputed scope</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>LV: inspector report finding some storm damage plus workman tile damage, inferior valley lead, crumbling mortar; absence of invoices for 2013, 2014 and 2015 claim repairs; concerns about 2012 invoice. Policyholder: roofer's report saying sagging caused by storm-driven water ingress; engineer's report confirming good construction, quality award, correct purlin spacing, leaks attributable to storm not structural deficiencies; claimed to have sent proof of repairs to LV but could not provide evidence to FOS; offer to obtain structural engineer's report not followed through</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; LV's initial settlement of ~£5,000 not disturbed; additional ~£21,000 quote not payable — policyholder failed to show damage was attributable to 2016 storm rather than cumulative unrepaired prior storm damage; LV's non-renewal decision also confirmed as LV's commercial prerogative; no award</t>
+        </is>
+      </c>
+      <c r="N35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P35" s="5" t="inlineStr">
+        <is>
+          <t>Where a policyholder has multiple prior settled storm claims paid in cash, the burden is on the policyholder to demonstrate those repairs were actually carried out before claiming for what may be cumulative deterioration; an engineer's report establishing general structural soundness and attributing leaks generally to storm does not establish Q3 for a specific additional claim scope where it does not identify which areas are leaking, the duration of problems, or the specific repair scope required; evidence offered but not provided to FOS cannot be considered; an insurer's non-renewal decision is a commercial decision FOS will not override</t>
+        </is>
+      </c>
+      <c r="Q35" s="5" t="inlineStr">
+        <is>
+          <t>Invoices or receipts demonstrating that prior claim cash settlements for 2013, 2014 and 2015 were used to carry out the agreed repairs; an expert report identifying which specific areas of the roof were leaking, how long problems had persisted, and the scope of repairs attributable to the 2016 storm as distinct from cumulative unrepaired prior damage</t>
+        </is>
+      </c>
+      <c r="R35" s="5" t="inlineStr">
+        <is>
+          <t>Mr M provided evidence of storm damage to roof generally but not that current damage was attributable to the 2016 storm specifically; LV had paid cash settlements for multiple prior claims (2012-2015); LV required invoices confirming repairs were carried out; only 2012 invoice provided and that raised concerns; FOS found it more likely than not that prior invoices were not sent to LV; if prior repairs were not carried out and damage accumulated, LV not required to pay for that cumulative deterioration; engineer's report confirmed structural soundness and attributed leaks generally to storm but did not identify specific leaking areas, duration, or repair scope — insufficient to establish Q3 for the additional claim; LV's initial £5,000 settlement not disturbed; non-renewal is LV's commercial decision.</t>
+        </is>
+      </c>
+      <c r="S35" s="5" t="inlineStr">
+        <is>
+          <t>For policyholders with a history of multiple storm claims paid in cash, require proof of completed repairs before paying further claims — the prior repair requirement is FOS-endorsed; where a policyholder submits a general expert opinion attributing leaks to storm damage but the report does not address which specific areas are leaking or the current repair scope, it is insufficient to establish Q3 for the disputed additional amount; document why prior invoices are inadequate or absent in decline reasoning</t>
+        </is>
+      </c>
+      <c r="T35" s="5" t="inlineStr">
+        <is>
+          <t>IF multiple_prior_settled_storm_claims AND policyholder_cannot_evidence_prior_repairs_completed THEN current_claim_may_be_declined_as_cumulative_unrepaired_damage; IF expert_report_attributes_leaks_generally_to_storm BUT does_not_identify_specific_leaking_areas_or_repair_scope THEN insufficient_to_establish_q3_for_additional_claim; IF prior_claims_settled_in_cash AND no_repair_invoices THEN require_proof_of_completed_repairs_before_paying_further_claims</t>
+        </is>
+      </c>
+      <c r="U35" s="4" t="inlineStr">
+        <is>
+          <t>DRN7021460.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="120" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>STORM-035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>DRN7244667</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Liverpool Victoria Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>2 Aug 2020</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Storm damage to tiled roof and internal ceiling declined; winds reached 41mph; LV's trusted provider inspection found damage not consistent with a one-off event and pre-existing; policyholder's independent report suggested tiles moved by high winds; FOS found Q1 failed — 41mph winds and low hourly rainfall do not constitute storm conditions</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Tiled roof — tiles reportedly moved by high winds allowing water ingress causing internal ceiling collapse; LV's trusted provider and review of independent report concluded damage was not consistent with a one-off storm event and appeared pre-existing and gradual</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>Weather records showed maximum winds of 41mph — below storm threshold; hourly rainfall not exceptional; LV's inspector found damage not consistent with a one-off event (pre-existing, gradual); independent report submitted by policyholder attributed damage to high winds but high winds at 41mph do not constitute storm conditions</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>LV: weather records showing 41mph winds; trusted provider inspection finding damage not consistent with one-off event and appearing pre-existing; LV's review of independent report finding damage not consistent with storm damage. Policyholder (represented by Mr A): independent report suggesting high winds moved tiles and rain entered; roofer said damage caused by weather conditions; workmen could not access roof during first visit due to wind; alleged further damage caused while awaiting repair</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; Q1 failed — winds 41mph below storm threshold and hourly rainfall not exceptional; storm conditions not established; damage more likely from gradual wear and tear and multiple causes; LV's decline confirmed as fair; no award</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P36" s="3" t="inlineStr">
+        <is>
+          <t>41mph winds without exceptional accompanying rainfall do not constitute storm conditions; storm conditions can exist without very strong winds only if accompanied by exceptional rainfall, hail, or snowfall — both wind and precipitation must be assessed together; workmen being unable to access a roof for safety reasons does not constitute evidence of storm conditions; strong winds are not the same as a storm; a roof in poor condition that cannot withstand normal weather does not give rise to a storm claim where storm conditions are not established</t>
+        </is>
+      </c>
+      <c r="Q36" s="3" t="inlineStr">
+        <is>
+          <t>Evidence of exceptional rainfall, hail, or snowfall concurrent with the 41mph winds; expert evidence establishing storm causation rather than pre-existing gradual deterioration</t>
+        </is>
+      </c>
+      <c r="R36" s="3" t="inlineStr">
+        <is>
+          <t>Q1 — weather records showed 41mph winds; FOS considers storm winds to be stronger; storm conditions can exist without very strong winds only if rainfall, hail, or snowfall is exceptional; hourly rainfall was not high; no evidence of storm conditions around the date of claim; Q1 answered no. Q2 and Q3 not considered. LV's inspector found damage not consistent with a one-off event (pre-existing, gradual); LV reviewed independent report and found damage not consistent with storm; roofer's opinion that tiles moved by high winds does not establish storm conditions; delay in repair did not alter the pre-existing damage finding.</t>
+        </is>
+      </c>
+      <c r="S36" s="3" t="inlineStr">
+        <is>
+          <t>When declining on sub-storm wind speeds, also document the precipitation levels — if both wind and rainfall are below storm thresholds Q1 is clearly answered no; being unable to access a roof due to wind is a workman safety consideration, not storm conditions evidence; where a policyholder's independent report attributes tile movement to high winds but does not establish storm conditions, the insurer can rely on its own inspector's pre-existing damage finding; once Q1 fails Q2 and Q3 need not be addressed</t>
+        </is>
+      </c>
+      <c r="T36" s="3" t="inlineStr">
+        <is>
+          <t>IF winds_41mph AND rainfall_not_exceptional AND no_exceptional_hail_or_snow THEN storm_q1 = no; IF storm_conditions_not_established THEN q2_and_q3_not_considered AND claim_fails; IF workmen_cannot_access_roof_due_to_wind THEN not_evidence_of_storm_conditions; IF independent_report_attributes_damage_to_high_winds_only AND high_winds_not_storm THEN report_does_not_establish_storm_q1</t>
+        </is>
+      </c>
+      <c r="U36" s="2" t="inlineStr">
+        <is>
+          <t>DRN7244667.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add STORM-036 to STORM-038 to Storm Case Database — complete
All 38 storm damage FOS cases processed. Storm database complete.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Storm_Case_Database.xlsx
+++ b/knowledge/case-databases/Storm_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U36"/>
+  <dimension ref="A1:U39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4278,6 +4278,321 @@
         </is>
       </c>
     </row>
+    <row r="37" ht="120" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>STORM-036</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>DRN8247030</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Royal &amp; Sun Alliance Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>26 Sep 2016</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Storm damage to roof of residential home declined; February 2016 claim; RSA's policy defined storm as exceptionally heavy rainfall usually accompanied by high winds; records showed no qualifying heavy rainfall and high winds a week earlier were not linked to physical roof damage; both RSA contractor inspections found poor design and workmanship at valley-gutter junction excluded under policy; policyholder also alleged defective 2013 RSA contractor repairs caused the leak but lacked independent expert evidence</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Roof valleys and boxed guttering junction — two RSA contractor inspections found a gap between roof and boxed guttering resulting from poor design and/or workmanship; external wall staining indicated gradual ongoing leak not a single storm event; 2013 RSA contractors denied their repairs caused the defect</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>No heavy rainfall meeting policy storm definition around the claim date; high winds about a week before not linked to any physical roof damage; both contractor inspections found poor design and workmanship at valley-gutter junction — excluded under policy clause covering 'any loss damage caused by or resulting from poor or faulty design, workmanship or materials'; external wall staining indicated gradual long-term leak not a single storm event; defective 2013 repairs claim unsupported by independent expert evidence</t>
+        </is>
+      </c>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>RSA: weather records showing no qualifying heavy rainfall; high winds one week before claim but no physical damage linked to them; two contractor inspection reports both finding poor design and workmanship at valley-gutter junction; original 2013 contractor denying liability; external wall staining. Mr B: property built 1998 with no evidence of leaks before 2013 claim; argued 2013 RSA contractors caused the defects; only evidence was contractor's own 2016 inspection report and photographs — no independent expert assessment of 2013 repair quality</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; Q1 failed — no heavy rainfall meeting RSA's policy storm definition; high winds a week before not linked to physical roof damage; Q2 also failed — both contractors found poor design and workmanship excluded under policy; defective repairs claim failed — no independent expert evidence that 2013 repairs were defective; internal damage also not storm-caused as leak was gradual; no award</t>
+        </is>
+      </c>
+      <c r="N37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P37" s="5" t="inlineStr">
+        <is>
+          <t>Storm defined as exceptionally heavy rainfall usually accompanied by high winds — absence of qualifying heavy rainfall around the claim date fails Q1; a policy exclusion for 'any loss damage caused by or resulting from poor or faulty design, workmanship or materials' defeats Q2 and Q3 where both contractor inspections identify poor design or workmanship as the cause; external wall staining indicating a gradual multi-year leak is negative evidence against storm causation; a defective contractor repairs claim requires independent expert evidence — the original contractor's denial of liability is not sufficient</t>
+        </is>
+      </c>
+      <c r="Q37" s="5" t="inlineStr">
+        <is>
+          <t>Weather records showing heavy rainfall meeting the policy storm definition around the claim date; independent expert evidence (separate from RSA's contractors) establishing that the 2013 repairs were defective and caused the current defect</t>
+        </is>
+      </c>
+      <c r="R37" s="5" t="inlineStr">
+        <is>
+          <t>Q1 — RSA's policy required exceptionally heavy rainfall usually accompanied by high winds; records showed no qualifying heavy rainfall around the claim date; very high winds occurred about a week before but no physical damage to roof was linked to them; Q1 failed. Q2 and Q3 — even if Q1 had passed, both RSA contractor inspections found poor design and workmanship at the valley-gutter junction (gap between roof and boxed guttering); policy excluded loss caused by poor or faulty design, workmanship or materials; Q2 also failed. External wall staining showed leak had been ongoing for some time not caused by a single storm. Defective repairs: only expert evidence was the contractor who carried out the 2013 repairs and their 2016 photos; contractor denied liability; no independent expert showed 2013 repairs were defective. Internal damage: no storm established and leak was gradual.</t>
+        </is>
+      </c>
+      <c r="S37" s="5" t="inlineStr">
+        <is>
+          <t>Where a policy defines storm as requiring exceptionally heavy rainfall, document weather records showing rainfall levels specifically — sub-storm rainfall is a standalone Q1 failure independent of wind speed; a faulty design or workmanship exclusion provides a dual basis for declining the claim if the storm analysis also fails; where a policyholder alleges defective insurer-arranged contractor repairs, the insurer should proactively commission an independent expert assessment to avoid an unsupported 'he said/she said' position at FOS</t>
+        </is>
+      </c>
+      <c r="T37" s="5" t="inlineStr">
+        <is>
+          <t>IF policy_storm_definition_requires_heavy_rainfall AND no_qualifying_rainfall_recorded THEN storm_q1 = no; IF policy_excludes_poor_design_or_workmanship AND contractor_inspections_find_poor_design_or_workmanship THEN q2_also_fails; IF policyholder_alleges_defective_contractor_repairs AND only_evidence_is_contractor_self_assessment THEN defective_repairs_claim_fails_for_lack_of_independent_expert_evidence</t>
+        </is>
+      </c>
+      <c r="U37" s="4" t="inlineStr">
+        <is>
+          <t>DRN8247030.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="120" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>STORM-037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>DRN8636254</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>21 Nov 2016</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Storm damage to roof of block of flats partially accepted; tiles dislodged and paid by Aviva; felt and battens underneath declined as wear and tear; residents association argued felt was punctured by dislodged tiles during storm; surveyor and FOS found felt and battens had rotted gradually over time — storm highlighted maintenance issue not caused it</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Roof tiles — dislodged by storm (accepted and paid by Aviva); felt and battens underneath — found crumbling and rotted gradually over time by Aviva's surveyor; storm highlighted pre-existing maintenance issue rather than causing felt and batten damage</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Block of flats</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Partial</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>Aviva's surveyor found felt and battens in poor state of repair, having rotted over a period of time; photographs showed felt crumbling and battens in poor condition consistent with gradual wear and tear not storm damage; storm highlighted an existing maintenance issue rather than causing the damage; policy covers one-off storm damage not gradual maintenance deterioration</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>Aviva: surveyor report finding felt and battens in poor state of repair, rotted over time, storm highlighted maintenance issue; photographs showing felt crumbling and battens in poor condition. Residents association B: argued felt was directly punctured by the storm-dislodged tiles; contended damage to felt and battens would not have occurred were it not for the storm</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; Aviva's partial acceptance of tile damage confirmed as correct; felt and battens decline confirmed — Q3 failed; surveyor and photographs showed gradual rot and deterioration not storm-caused damage; Aviva's decision to decline felt and battens confirmed as reasonable; no further award</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P38" s="3" t="inlineStr">
+        <is>
+          <t>Q3 — damage to felt and battens that shows crumbling and rot consistent with gradual deterioration over time is not caused by a storm even where tiles above were storm-damaged; policy covers one-off storm incidents not maintenance deterioration that comes to light at the time of a storm; damage to felt and battens is not typical of storm damage (though possible in certain circumstances) — where photographs show rot and crumbling the Q3 answer is no; an insurer can accept storm damage to tiles while simultaneously declining felt and battens on wear and tear grounds where the two damage types have different causation</t>
+        </is>
+      </c>
+      <c r="Q38" s="3" t="inlineStr">
+        <is>
+          <t>Expert or photographic evidence showing the felt was intact immediately before the storm and was specifically punctured or torn by the dislodged tiles rather than already rotted</t>
+        </is>
+      </c>
+      <c r="R38" s="3" t="inlineStr">
+        <is>
+          <t>Q1 — Aviva accepted storm; yes. Q2 — tile damage accepted; damage to felt and battens not typical of storm damage but FOS accepted it could happen in certain circumstances. Q3 — Aviva's surveyor said felt and battens in poor state, rotted over time; storm highlighted maintenance issue, did not cause the damage; FOS reviewed photographs which showed felt crumbling and battens in poor condition — consistent with gradual wear and tear over time not damage from a single storm; Q3 answered no for felt and battens. FOS noted it was not considering the claim for internal damage (which was not pursued as the flat occupier sadly passed away).</t>
+        </is>
+      </c>
+      <c r="S38" s="3" t="inlineStr">
+        <is>
+          <t>When accepting partial storm damage (tiles), assess felt and battens separately under Q3 — their condition may reflect gradual deterioration even where tiles above were storm-damaged; document the surveyor's specific findings on felt and batten condition with photographs to support a partial decline; where photographs show crumbling felt and rotted battens, Q3 for that element fails regardless of what caused tile damage above; a one-off storm does not cause rot — rot is definitionally gradual</t>
+        </is>
+      </c>
+      <c r="T38" s="3" t="inlineStr">
+        <is>
+          <t>IF tiles_accepted_as_storm_damaged AND felt_and_battens_show_crumbling_and_rot THEN felt_and_battens_q3 = no AND partial_decline_reasonable; IF surveyor_finds_gradual_rot_in_felt_and_battens THEN storm_not_main_cause_of_felt_and_batten_damage; IF damage_element_shows_gradual_deterioration THEN assess_q3_independently_from_other_accepted_storm_damage_elements</t>
+        </is>
+      </c>
+      <c r="U38" s="2" t="inlineStr">
+        <is>
+          <t>DRN8636254.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="120" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>STORM-038</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>DRN8660161</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Zurich Insurance PLC</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>29 Feb 2016</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Three-claim complaint: subsidence 2006 declined (no evidence); storm damage 2013 declined (gradual deterioration, no AD cover for internal damage); storm damage 2015 declined (same roofs in poor condition, storm not main cause); policyholder's specific storm event claims unsupported by evidence; surveyor reports showed 60-80 year old main roof in very poor condition</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Main roof and flat roof of residential home — surveyor reports for both 2013 and 2015 claims showed roofs in very poor state of repair; main roof 60-80 years old with very worn mortar and nails, temporary repairs made; flat roof old for its type; 2015 roofer report noted materials had blown off but FOS found storm merely highlighted pre-existing poor condition</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J39" s="5" t="inlineStr">
+        <is>
+          <t>Subsidence 2006: loss adjuster found no evidence of subsidence and no contrary evidence provided. Storm 2013 and 2015: main roof estimated 60-80 years old with very worn mortar and nails; flat roof old for its type; surveyor reports for both claims showed poor condition due to lack of maintenance; policyholder claimed greenhouse glass blown onto roof (2013) and branch blown against chimney (2015) but neither was supported by evidence; storm highlighted poor condition rather than causing damage; gradually-occurring maintenance damage excluded under policy</t>
+        </is>
+      </c>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>Zurich: loss adjuster letter (2006) finding no subsidence evidence; surveyor reports for both 2013 and 2015 claims showing roofs in very poor condition due to lack of maintenance; 2015 roofer report noting materials had blown off (accepted by FOS as possible but not determinative of causation). Miss J: claimed roofs had been maintained (contradicted by photos and reports); claimed 2013 damage caused by storm-blown greenhouse glass onto roof; claimed 2015 chimney damaged by storm-blown branch; claimed roof damage caused by subsidence — no evidence provided for any of these specific events</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold on any head; subsidence claim failed — no evidence provided; both storm claims failed — surveyor reports showed roofs in very poor condition from lack of maintenance; specific storm event claims (greenhouse glass, blown branch) unsupported by evidence; storm highlighted poor condition rather than causing damage; gradually-occurring maintenance damage excluded; 2013 internal damage correctly declined as no AD cover; 2015 internal damage — no evidence of any internal damage; no award</t>
+        </is>
+      </c>
+      <c r="N39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P39" s="5" t="inlineStr">
+        <is>
+          <t>Q3 failed for both storm claims — roofs in very poor condition from lack of maintenance (main roof 60-80 years old, mortar and nails very worn) with storm merely highlighting the pre-existing condition; a policyholder's unsupported assertion of a specific storm event (greenhouse glass, blown branch) is not sufficient to establish storm causation; gradually-occurring damage from lack of maintenance is excluded under policy; absence of AD cover correctly prevents recovery of internal damage under the 2013 policy; where AD cover exists in 2015 but no evidence of internal damage is presented the claim also fails</t>
+        </is>
+      </c>
+      <c r="Q39" s="5" t="inlineStr">
+        <is>
+          <t>Evidence supporting the specific 2013 storm event (greenhouse glass blown onto roof) and 2015 event (branch blown against chimney); evidence that roofs were in good condition and maintained before the storms; evidence of internal damage in 2015</t>
+        </is>
+      </c>
+      <c r="R39" s="5" t="inlineStr">
+        <is>
+          <t>Subsidence 2006: loss adjuster letter found no evidence; Miss J provided nothing to contradict — not upheld. Storm 2013 and 2015: storms occurred around both claim dates; Miss J claimed greenhouse glass blown onto roof (2013) — nothing to support this; claimed branch blown against chimney (2015) — nothing to support this; surveyor reports for both claims showed roofs in very poor condition — main roof 60-80 years old, mortar and nails very worn, temporary repairs made, flat roof old for its type; Miss J claimed roofs were maintained but photos and reports contradicted this; 2015 roofer noted materials had blown off — FOS accepted this may have happened but concluded storm just highlighted poor condition rather than causing damage; Q3 no for both claims; gradually-occurring damage from lack of maintenance excluded; 2013 internal damage: correctly declined as no AD cover; 2015 internal damage: AD cover existed but no evidence of any internal damage presented.</t>
+        </is>
+      </c>
+      <c r="S39" s="5" t="inlineStr">
+        <is>
+          <t>Where a policyholder makes multiple claims over multiple years with roofs consistently found to be in poor condition, the accumulation of surveyor reports showing unmaintained roofs is strong Q3 evidence; a policyholder's assertion of a specific storm trigger event (object blown onto roof, branch impact) must be supported by evidence — unsupported assertions will not displace consistent surveyor findings of general poor condition; when AD cover is absent, decline internal damage at first handling with a clear explanation to avoid a separate complaint</t>
+        </is>
+      </c>
+      <c r="T39" s="5" t="inlineStr">
+        <is>
+          <t>IF surveyor_reports_across_multiple_claims_show_poor_roof_condition AND policyholder_claims_specific_storm_trigger_unsupported THEN storm_q3 = no_for_all_claims; IF gradually_occurring_damage_from_lack_of_maintenance THEN excluded_under_policy; IF no_ad_cover AND internal_damage_claimed THEN internal_damage_declined_correctly; IF ad_cover_exists AND no_evidence_of_internal_damage THEN internal_damage_claim_also_fails</t>
+        </is>
+      </c>
+      <c r="U39" s="4" t="inlineStr">
+        <is>
+          <t>DRN8660161.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>